<commit_message>
Re-translate 344 stored Korean titles with nuclear terminology
MyMemory output had systematic term errors (열유압, 조약돌층, 반응기, stray ¶).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sHSCbWkWUBv2qJdcCnH5x
</commit_message>
<xml_diff>
--- a/outputs/nuclear-literature-database.xlsx
+++ b/outputs/nuclear-literature-database.xlsx
@@ -1364,7 +1364,7 @@
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>UZrHx 연료 반응기에서의 수소 동역학 및 그 영향에 대한 다중 물리학 분석</t>
+          <t>UZrHx 핵연료 원자로에서 수소 거동 동역학 및 그 영향에 대한 다중물리 해석</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>비선형 진동에 의해 유도된 PWR 연료봉의 비대칭 격자-봉 프레팅 마모에 대해</t>
+          <t>비선형 진동에 의한 PWR 핵연료봉의 비대칭 지지격자-연료봉 프레팅 마모</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>공기 중 라돈 및 토론 붕괴 생성물의 잠재적 알파 에너지 농도를 결정하기 위한 통합 방법</t>
+          <t>공기 중 라돈 및 토론 붕괴생성물의 잠재 알파에너지 농도 결정을 위한 적분법</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>400MWth 자연 순환 납 냉각 반응기와 결합된 초임계 이산화탄소 재압축 브레이튼 사이클 에너지 컨버터의 동적 모델링 및 시뮬레이션</t>
+          <t>400 MWth 자연순환 납냉각 원자로와 연계된 초임계 이산화탄소 재압축 브레이튼 사이클 에너지 변환기의 동적 모델링 및 모의</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>디지털 팬텀을 사용하는 소형 플래시 방사선 치료 장치를 위한 X선 유도 음향 선량 측정의 시뮬레이션 연구</t>
+          <t>디지털 팬텀을 이용한 소형 FLASH 방사선치료 장치의 X선 유도 음향 선량 측정 모의 연구</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>히트 파이프 원자로 핵 에너지 시스템을 위한 3D 중성자-수송 기반 시스템 분석 코드 개발</t>
+          <t>히트파이프 원자로 원자력 에너지 계통을 위한 3차원 중성자 수송 기반 계통해석 코드 개발</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>TIME PETRI NET을 기반으로 SMR의 Main Control Room에서 작업자 협업을 위한 모델링</t>
+          <t>시간 페트리넷 기반 SMR 주제어실 운전원 협업 모델링</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>공간을 사용하는 혁신적인 SMR에서 다발성 고장 사고가 발생한 나선형 코일 스팀 발생기 튜브 파열 분석</t>
+          <t>SPACE를 이용한 혁신형 SMR의 다중고장 동반 나선형 코일 증기발생기 전열관 파단사고 해석</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>단일 루프 수동 냉각을 사용한 셧다운 냉각 로카 중 비대칭 루프 씰 클리어링 및 개질: ATLAS 적분 효과 테스트 및 MARS-KS 평가</t>
+          <t>단일루프 피동냉각 조건의 정지냉각 LOCA 시 비대칭 루프실 제거 및 재형성: ATLAS 종합효과시험 및 MARS-KS 평가</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>필리핀 바탄 원자력 발전소의 잠재적 재가동을 위한 대기 분산 모델링 및 방사선 환경 영향 평가</t>
+          <t>필리핀 바탄 원자력발전소 재가동 가능성에 대한 대기확산 모델링 및 방사선 환경영향평가</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>신규 나선형 인쇄 회로 열교환기의 실험적 및 수치적 열-유압 성능 분석</t>
+          <t>신형 나선형 인쇄기판형 열교환기의 열수력 성능에 관한 실험 및 수치해석</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>200MWt 선박용 용융 염화물 고속 반응기를 위한 개선된 코어 설계 및 통합 백엔드 연료 사이클 방식</t>
+          <t>200 MWt 선박용 용융염화물 고속로의 개선된 노심 설계 및 통합 후행 핵연료주기 방안</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>고속 스펙트럼 리튬 냉각 우주 원자로를 위한 퍼지 예측 제어 및 칼만 필터를 기반으로 한 코어 전력 제어 조사</t>
+          <t>고속 스펙트럼 리튬냉각 우주용 원자로의 퍼지 예측제어 및 칼만 필터 기반 노심출력 제어 연구</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>공기 중 감마선 분광 데이터에 대한 이상 인식 레벨링 알고리즘</t>
+          <t>항공 감마선 분광 데이터를 위한 이상치 인지 레벨링 알고리즘</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>압연 조건에서 소형 꽃잎 모양의 연료봉 번들 채널의 자연 순환 특성</t>
+          <t>요동 조건에서 소형 꽃잎형 핵연료봉 다발 유로의 자연순환 특성</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>소형 모듈형 반응기용 다중 코일 평행 나선형 코일 튜브의 밀도파 진동에 관한 연구</t>
+          <t>소형모듈원자로용 다중 코일 병렬 나선형 전열관의 밀도파 진동 연구</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>저전력 조건에서 번들 재홍수 중 DRACCAR 예측 능력 평가: 체계적인 불확실성 및 민감도 분석</t>
+          <t>저출력 조건 핵연료다발 재관수 시 DRACCAR 예측 성능 평가: 체계적 불확실성 및 민감도 분석</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>용융염 천연 순환 루프에서 국소 가열 효과의 실험적 유동 시각화 및 열-유압 특성 분석</t>
+          <t>용융염 자연순환 루프에서 국부 가열 효과의 유동 가시화 실험 및 열수력 특성 규명</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>고유동 2상 유동 및 연행 메커니즘 조사</t>
+          <t>고유속 2상유동 및 비말동반 메커니즘 연구</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>EP823-SH 스틸 클래딩의 내부 표면에 전착 크롬 코팅의 미세 구조 및 수소 함량</t>
+          <t>EP823-SH 강 피복관 내면 전착 크롬 코팅의 미세조직 및 수소 함량</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>ASME 섹션 III과 체코 NTD A.S.I. 섹션 III: 도메인 및 구성 요소 해결 평가 간의 조항 수준 구조 정렬</t>
+          <t>ASME Section III와 체코 NTD A.S.I. Section III 간 조항 수준 구조적 대응: 분야 및 기기별 평가</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>VVER-1200에 대한 잠재적 사고 내성 연료 구성의 비교 중성 성능 평가</t>
+          <t>VVER-1200용 사고저항성핵연료(ATF) 후보 구성의 중성자 성능 비교 평가</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>한국 규제 프레임워크에 대한 검사 성숙도 수준 모델 개발 및 소비 연료 건식 저장 시설에 적용</t>
+          <t>국내 규제체계를 위한 검사 성숙도 수준 모델 개발 및 사용후핵연료 건식저장시설 적용</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>EXL-50U 구형 토카막 장치용 토로이드 필드 자석 전원 공급 장치의 엔지니어링 설계 및 검증</t>
+          <t>EXL-50U 구형 토카막 장치의 토로이달 자장 코일 전원장치 공학설계 및 검증</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>광학 및 방사선 차폐 응용 분야를 위한 B                    &lt;sub&gt;2&lt;/sub&gt; O                    &lt;sub&gt;3&lt;/sub&gt; -TiO                    &lt;sub&gt;2 -BaO-ZnO-CeO 2&lt;/sub&gt; 안경의 제작 및 특성 분석                    &lt;sub&gt;&lt;/sub&gt;</t>
+          <t>광학 및 방사선 차폐용 B2O3-TiO2-BaO-ZnO-CeO2 유리의 제조 및 특성 분석</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>원자로 부품의 자동 결함 감지를 위한 지식 기반 설명 가능한 AI</t>
+          <t>원자로 구성품 자동 결함 탐지를 위한 지식 기반 설명가능 AI</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>중국 원자력 발전소의 운영 사건을 분류하고 분석하기 위한 인간-장비-사회 (Human-Equipment-Society, HES) 프레임워크</t>
+          <t>중국 원자력발전소 운전사건 분류 및 분석을 위한 인간-설비-사회(HES) 프레임워크</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>원자력 발전소 현장에서 방사성 핵종을 운반하기 위한 ERA5 데이터를 기반으로 불리한 기상 조건을 추정합니다.</t>
+          <t>ERA5 데이터 기반 원자력발전소 부지로부터 방사성핵종 이동에 불리한 기상조건 추정</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>다수의 알려지지 않은 소스로부터의 방사선 필드의 3D 재구성을 위한 하이브리드 신경-복셀 물리학-제약 프레임워크</t>
+          <t>미지의 다중 선원으로부터 방사선장 3차원 재구성을 위한 신경망-복셀 하이브리드 물리제약 프레임워크</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -4132,7 +4132,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>NekRS 스펙트럼 요소 Navier–Stokes 솔버에 대한 몰입 경계 방법</t>
+          <t>NekRS 스펙트럴 요소 Navier–Stokes 해석기를 위한 가상경계법</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>방사성 대기 방출 하에서의 비상 계획 구역 평가를 위한 신뢰성 기반 프레임워크</t>
+          <t>방사성물질 대기 방출 시 비상계획구역 평가를 위한 신뢰도 기반 프레임워크</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>원자력 안전 계산을 위한 딥러닝 기법 적용, LBLOCA 시나리오 분석</t>
+          <t>원자력 안전 계산을 위한 딥러닝 기법 적용: LBLOCA 시나리오 해석</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>납-비스무트 공융에서 Si-containing ferritic/martensitic steel의 산화 거동에 대한 전기화학적 임피던스 분광학 조사</t>
+          <t>납–비스무트 공정 내 Si 함유 페라이트/마르텐사이트강 산화 거동의 전기화학 임피던스 분광 연구</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4492,7 +4492,7 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>원자력 산업 제어 시스템의 제어기 영역 네트워크에 대한 비감독 이상 탐지 방법</t>
+          <t>원자력 산업제어계통 CAN(Controller Area Network)을 위한 비지도 이상탐지 방법</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>반응기 냉각수 펌프에서 입구 경계 조건 및 난류 모델이 압력 맥동 예측에 미치는 영향</t>
+          <t>원자로냉각재펌프 압력맥동 예측에 대한 입구 경계조건 및 난류모델의 영향</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>MURR 고검정 저농축 우라늄 연료 요소와 설계 실증 요소 조사 열-기계 분석 예측 비교</t>
+          <t>MURR HALEU 핵연료 요소와 설계실증 요소의 조사 열-기계 해석 예측 비교</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -4774,7 +4774,7 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Ac-225의 원자로 기반 생산 및 불순물 제어를 위한 중성자 스펙트럼 최적화</t>
+          <t>원자로 기반 Ac-225 생산 및 불순물 제어를 위한 중성자 스펙트럼 최적화</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>이온화 방사선에 대한 B                    &lt;sub&gt;2&lt;/sub&gt; O                    &lt;sub&gt;3 -Na&lt;/sub&gt;                    &lt;sub&gt;2&lt;/sub&gt; O-ZnO-CaO-Eu                    &lt;sub&gt;2&lt;/sub&gt; O                    &lt;sub&gt;3&lt;/sub&gt; 유리 시스템의 방사선 차폐 성능</t>
+          <t>B2O3-Na2O-ZnO-CaO-Eu2O3 유리계의 전리방사선 차폐 성능</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>기관 구조, 소유권 모델 및 원주민 지역 사회에서 마이크로 반응기의 경제적 영향</t>
+          <t>원격지 원주민 공동체 초소형원자로의 제도적 구조, 소유 모델 및 경제적 영향</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>위치 조건 하에서 Cr-코팅 지르칼로이-4 클래딩에서 계면 안정성 및 균열 유발 응집력 저하에 대한 수치 조사</t>
+          <t>LOCA 조건에서 Cr 코팅 지르칼로이-4 피복관의 계면 안정성 및 균열 유발 응집 열화 수치해석</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>UDF-강화 CFD 모델을 통한 해양 조건 하에서의 LBE-냉각 고속 원자로 어셈블리에서의 열-유압 거동 수치 조사</t>
+          <t>UDF 강화 CFD 모델을 이용한 해양 조건에서 LBE 냉각 고속로 집합체의 열수력 거동 수치해석</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>〈En〉 = 3 MeV에서 237Np (n, f) 반응으로부터의 프롬프트 중성자 스펙트럼</t>
+          <t>〈En〉=3 MeV에서 237Np(n,f) 반응의 즉발중성자 스펙트럼</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5348,7 +5348,7 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>언덕 지형의 방사성 플루토늄 에어로졸의 소규모 증착 거동</t>
+          <t>구릉 지형에서 방사성 플루토늄 에어로졸의 소규모 침적 거동</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>180 °C 고온의 물과 교대로 430 °C 증기/180 °C 물 환경에서 316 L의 산화물 진화</t>
+          <t>180 °C 고온수 및 430 °C 증기/180 °C 물 교번 환경에서 316L의 산화막 변화</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>핵 법의학의 글로벌 연구 동향: 참고문헌 검토</t>
+          <t>핵감식 분야의 전 세계 연구 동향: 계량서지학적 고찰</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>무인 항공기 위협에 대한 핵 시설의 물리적 보호: 식별 시기의 제약에 따른 성능 제한</t>
+          <t>무인 항공 위협에 대한 원자력시설 물리적 방호: 식별 시간 제약 하의 성능 한계</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5726,7 +5726,7 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>필리핀 원자력 연구소 소유의 레거시                    &lt;sup&gt;226&lt;/sup&gt; Ra 소스의 지속적인 보관에 대한 소유권 이전의 질적 비용-편익 평가</t>
+          <t>필리핀원자력연구소 보유 노후 226Ra 선원의 소유권 이전 대 계속 저장에 대한 정성적 비용편익 평가</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>오염 제거 현장과 관련된 이재민의 선택 행동은 대피에 어떤 영향을 미칩니까? — 중국의 원자력 발전소 사례 연구</t>
+          <t>제염소 선택 행태가 대피에 미치는 영향 — 중국 원자력발전소 사례 연구</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>원자력 발전소 운영 의사 결정을 지원하기 위한 장애 트리 분석을 위한 효율적인 방법</t>
+          <t>원자력발전소 운전 의사결정 지원을 위한 효율적 고장수목 분석 방법</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>200kW 수성 균질 반응기에서 작동 안정성을 위한 주요 결정 요인 식별</t>
+          <t>200 kW 수용액 균질로의 운전 안정성 핵심 결정인자 규명</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>MRI 스캐너를 사용하여 유동-파편 상호 작용 및 PWR 필터 막힘 동작의 CFD 등급 측정</t>
+          <t>MRI 스캐너를 이용한 유동-이물질 상호작용 및 PWR 필터 막힘 거동의 CFD급 측정</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6188,7 +6188,7 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>심각한 사고 시 핵 선박 침투 노즐의 변형 및 파단 모델링: 파트 I – 합금 600 모델링</t>
+          <t>중대사고 시 원자로용기 관통 노즐의 변형 및 파단 모델링: 제1부 – Alloy 600 모델링</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>심각한 사고 시 핵 선박 침투 노즐의 변형 및 파단 모델링: 파트 II – 합금 82 모델링 및 OLHF 테스트 데이터와의 비교</t>
+          <t>중대사고 시 원자로용기 관통 노즐의 변형 및 파단 모델링: 제2부 – Alloy 82 모델링 및 OLHF 시험 데이터와의 비교</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6376,7 +6376,7 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>해체 중 냉각수 접촉 인터페이스에서 CRUD 소스 용어의 중요성 검토</t>
+          <t>해체 중 냉각재 접촉 계면에서 CRUD 선원항의 중요성 검토</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>조약돌층 고온 가스냉각 반응기용 3차원 열유압코드 개발 및 적용</t>
+          <t>페블베드 고온가스로용 3차원 열수력 코드 개발 및 적용</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>스털링형 히트 파이프 반응기 시스템의 다중 물리학 결합 열-전기 성능 분석</t>
+          <t>스털링형 히트파이프 원자로 계통의 다중물리 연계 열-전기 변환 성능 해석</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>OPR-1000의 활성화 분석을 사용한 샘플링 전략 개발을 위한 불확실성 인식 슈퍼픽셀 세분화 및 베이시안 최적화</t>
+          <t>OPR-1000 방사화 분석을 이용한 시료채취 전략 수립을 위한 불확실성 고려 슈퍼픽셀 분할 및 베이지안 최적화</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>향상된 광학 기능과 감마선 차폐 특성을 위해 Eu3 + 및 Ba2 + 로 엔지니어링된 ZnO가 풍부한 붕산염-티타네이트 유리</t>
+          <t>광학 특성 및 감마선 차폐 성능 향상을 위해 Eu3+ 및 Ba2+를 첨가한 ZnO 고함량 붕산염-티탄산염 유리</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -6846,7 +6846,7 @@
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>증기 응축 공정의 VOF 방법 및 시뮬레이션을 위한 다층 증기-액체 상 변화 모델 개발</t>
+          <t>VOF 방법을 위한 다층 증기-액체 상변화 모델 개발 및 증기 응축 과정 모의</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -6940,7 +6940,7 @@
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>UO2 분말 감마 분광법에서의 자체 감쇠 특성 분석: 벌크 핵 물질의 질량 및 농축 정량화를 위한 매트릭스 독립 분석법 개발 ¶</t>
+          <t>UO2 분말 감마 분광분석의 자기감쇠 특성 규명: 벌크 핵물질의 질량 및 농축도 정량을 위한 매질 독립 분석법 개발</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>MSRE에서 열-유압 모델 단순화가 정상 상태 온도 분포에 미치는 영향</t>
+          <t>MSRE 정상상태 온도분포에 대한 열수력 모델 단순화의 영향</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -7128,7 +7128,7 @@
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>초음파 나노 결정 표면 개질 (UNSM) 에 의해 처리된 민감화된 304H 스테인리스 스틸의 미세조직 및 부식 거동에 가해지는 하중의 영향</t>
+          <t>초음파 나노결정 표면개질(UNSM) 처리된 예민화 304H 스테인리스강의 미세조직 및 부식 거동에 대한 인가 하중의 영향</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7222,7 +7222,7 @@
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>증기 발생기의 전-영역 열-유압 분석을 위한 결합된 3차원 다공성-매체 및 드리프트-플럭스 모델</t>
+          <t>증기발생기 전 영역 열수력 해석을 위한 3차원 다공성매질-표류유속 연계 모델</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7316,7 +7316,7 @@
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>붕산 용액으로부터 세슘과 루비듐의 분리를 위한 칼륨 구리 헥사시아노페레이트 (II) 의 합성 및 사용</t>
+          <t>붕산 용액으로부터 세슘 및 루비듐 분리를 위한 칼륨 구리 헥사시아노철산염(II)의 합성 및 활용</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7410,7 +7410,7 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>A Comparative Molecular Dynamics Study of Pre-existing Point Defect-Induced Tensile Strength Loss in Single Crystal Ni and NiCr</t>
+          <t>단결정 Ni 및 NiCr에서 기존 점결함에 의한 인장강도 저하의 분자동역학 비교 연구</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7598,7 +7598,7 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>MCNPX2.7을 통한 NuScale SMR 코어 검증 및 천연 가돌리늄 이외의 대체 연소 가능 흡수체 평가</t>
+          <t>MCNPX2.7을 이용한 NuScale SMR 노심 검증 및 천연 가돌리늄 대체 가연성흡수체 평가</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>가압수형 원자로에서 연료봉 클래딩의 마모 거동에 대한 수치 조사</t>
+          <t>가압경수로 핵연료 피복관의 프레팅 마모 거동 수치해석</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -7786,7 +7786,7 @@
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>고속 반응기에서 제어 로드 값과 배가 시간 비교: ENDF/B-VIII.0 및 JEFF-3.3을 사용한 정적 및 동적 뱀 2 시뮬레이션</t>
+          <t>고중성자속 원자로의 제어봉 가치 및 배가시간 비교: ENDF/B-VIII.0 및 JEFF-3.3을 이용한 정적·동적 Serpent 2 모의</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>방사성 폐기물 처리를 위한 점토 기반 장벽의 환경 성능: 포르투갈 지질 물질과의 관련성 검토</t>
+          <t>방사성폐기물 처분용 점토 기반 방벽의 환경 성능: 포르투갈 지질 재료와 관련한 고찰</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -7966,7 +7966,7 @@
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>풍계리 미사일 충격 및 장시간 폭발 하중을 받는 원자력 발전소에서 특수 도어의 보호 성능에 대한 실험적 및 수치적 연구</t>
+          <t>비산물 충돌 및 장시간 폭발하중을 받는 원자력발전소 특수문의 방호 성능에 관한 실험 및 수치해석 연구</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>납-비스무스 공융 루프에서의 산소 제어에 대한 연구</t>
+          <t>납–비스무트 공정 루프에서의 산소 제어 연구</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>온도 의존성 프레팅 시뮬레이션된 PWR 1차 물에서 지르코늄 합금 클래딩 튜브의 마모</t>
+          <t>모의 PWR 1차계통수 환경에서 지르코늄 합금 피복관의 온도 의존 프레팅 마모</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8248,7 +8248,7 @@
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>PWR First-cycle Loading-Pattern Optimization을 위한 Deep Generative Model 및 Bayesian Optimization Scheme</t>
+          <t>PWR 초기노심 장전모형 최적화를 위한 심층생성모델 및 베이지안 최적화 기법</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>형태학적 가변성을 고려한 수소화물 함유 SNF 클래딩에 대한 골절 매개변수 추정에 대한 다목적 접근법</t>
+          <t>형상 변동성을 고려한 수소화물 함유 사용후핵연료 피복관 파괴 변수 추정을 위한 다목적 접근법</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>용융염 반응기 쉘-튜브 열교환기에서 지연된 중성자 전구체의 체류 시간 분포</t>
+          <t>용융염원자로 쉘-튜브 열교환기 내 지발중성자 선행핵 체류시간 분포</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>서브채널 모듈러 분석 프로그램의 검증 및 민감도 분석</t>
+          <t>부수로 모듈형 해석 프로그램의 검증 및 민감도 분석</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>1차 마그네슘 생산과 원자력의 통합을 위한 에너지 요구 및 해수 추출 접근법 분석</t>
+          <t>원자력과 1차 마그네슘 생산의 연계를 위한 에너지 수요 및 해수 추출 방식 분석</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>사고 허용 연료 클래딩의 적용에서 칸탈 APMT 페라이트 합금의 레이저 빔 용접 특성 및 미세 구조 특성</t>
+          <t>사고저항성핵연료 피복관 적용을 위한 Kanthal APMT 페라이트계 합금의 레이저빔 용접 특성 및 미세조직 분석</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>2500–2800 °C 범위에서 열처리된 TRISO 입자에서 SiC 층의 미세 구조 및 기계적 특성</t>
+          <t>2500–2800 °C 범위에서 열처리된 TRISO 입자 SiC 층의 미세조직 및 기계적 특성</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -8906,7 +8906,7 @@
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>공기 중에 스팀 응축을 위한 서브 그리드 기반 분석 벽 기능</t>
+          <t>공기 존재 하 증기 응축을 위한 부격자 기반 해석적 벽함수</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -9000,7 +9000,7 @@
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>알칼리성 폐수에서 효율적인 우라늄 제거를 위한 할로겐성 박테리아 유래 생체흡착제: 제조, 성능 및 메커니즘</t>
+          <t>알칼리성 폐수로부터 효율적 우라늄 제거를 위한 호염성 세균 유래 생체흡착제: 제조, 성능 및 메커니즘</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>나선형 코일형 튜브에 대해 국부적으로 업데이트된 특성을 사용하는 시스템 코드 지향 2상 마찰 압력 강하 상관관계의 개발 및 검증</t>
+          <t>국부 갱신 물성치를 이용한 계통코드용 나선형 코일관 2상 마찰압력강하 상관식 개발 및 검증</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -9188,7 +9188,7 @@
       </c>
       <c r="C86" s="9" t="inlineStr">
         <is>
-          <t>소아 방사선 치료에서 CT 기반 HU-RED 보정을 위한 확립된 참조 팬텀에 대한 새로운 다중 조직 의인화 소아 머리 팬텀의 개발 및 벤치마킹</t>
+          <t>소아 방사선치료 CT 기반 HU-RED 교정을 위한 신규 다조직 인체형 소아 두부 팬텀 개발 및 기존 기준 팬텀 대비 벤치마킹</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -9282,7 +9282,7 @@
       </c>
       <c r="C87" s="9" t="inlineStr">
         <is>
-          <t>물리 정보 신경망을 사용한 희소 측정 기반 3차원 방사선 필드 재구성</t>
+          <t>물리정보신경망을 이용한 희소 측정 기반 3차원 방사선장 재구성</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C89" s="9" t="inlineStr">
         <is>
-          <t>측면 양력에 중점을 둔 파일럿 규모의 버블 기둥에서 균질 흐름 체제의 계산 모델링 기능 및 제한 사항</t>
+          <t>파일럿 규모 기포탑 균질 유동영역 전산 모델링의 능력과 한계: 횡방향 양력을 중심으로</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -9634,7 +9634,7 @@
       </c>
       <c r="C91" s="9" t="inlineStr">
         <is>
-          <t>항우연 모드 사용 시 광자 계수 X선 영상에서 빔 경화 및 검출기 응답 기능 보정의 영향</t>
+          <t>반동시계수 모드 사용 시 광자계수 X선 영상에서 빔 경화 및 검출기 응답함수 보정의 영향</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -9728,7 +9728,7 @@
       </c>
       <c r="C92" s="9" t="inlineStr">
         <is>
-          <t>LiF-BeF2-UF4-ZrF4 용융염에서 Mo의 국소 구조 및 초기 단계 응집 거동</t>
+          <t>LiF-BeF2-UF4-ZrF4 용융염에서 Mo의 국부 구조 및 초기 응집 거동</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -9822,7 +9822,7 @@
       </c>
       <c r="C93" s="9" t="inlineStr">
         <is>
-          <t>I&amp;amp;C Focused System Dynamics를 사용하여 원자력 발전소를 대상으로 하는 사이버 공격 시나리오 개발</t>
+          <t>계측제어 중심 시스템 다이내믹스를 이용한 원자력발전소 대상 사이버공격 시나리오 개발</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -9916,7 +9916,7 @@
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>원자력 시설에서 방사능 방출이 환경에 미치는 영향을 평가하기 위한 시뮬레이션 기반 인공 지능 프레임워크: 실제 사례 연구</t>
+          <t>원자력시설 방사성물질 방출의 환경영향 평가를 위한 모의 기반 인공지능 프레임워크: 실제 사례 연구</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -10010,7 +10010,7 @@
       </c>
       <c r="C95" s="9" t="inlineStr">
         <is>
-          <t>배플 위치가 용액 배출에서 생성된 에어로졸의 분포 특성에 미치는 영향</t>
+          <t>용액 분출로 생성된 에어로졸의 분포 특성에 대한 배플 위치의 영향</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="C96" s="9" t="inlineStr">
         <is>
-          <t>납-비스무트-유텍틱 루프를 위한 고-레이놀즈 k-ω-kθ-θθ 모델 및 하이브리드 분해능 시뮬레이션 방법 개발</t>
+          <t>납-비스무트 공정 루프를 위한 고레이놀즈수 k–ω–kθ–ϵθ 모델 및 혼합 해상도 모의 방법 개발</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -10198,7 +10198,7 @@
       </c>
       <c r="C97" s="9" t="inlineStr">
         <is>
-          <t>안전장치 기술의 운용 준비성을 강화하기 위한 핵 비확산을 위한 AI 기반 스펙트럼 분석</t>
+          <t>안전조치 기술의 운용 준비태세 강화를 위한 핵비확산용 AI 기반 스펙트럼 분석</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -10292,7 +10292,7 @@
       </c>
       <c r="C98" s="9" t="inlineStr">
         <is>
-          <t>U-50Zr 나선형 십자형 연료의 성능 분석을 위한 중성자-열-유체 구조 커플링 방법론 개발</t>
+          <t>U-50Zr 나선형 십자형 핵연료 성능해석을 위한 중성자–열–유체–구조 연계 방법론 개발</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -10386,7 +10386,7 @@
       </c>
       <c r="C99" s="9" t="inlineStr">
         <is>
-          <t>MARVEL 마이크로 반응기에서 U-ZrH 및 MOX 연료 막대의 정상 작동 및 로카 성능에 대한 연료 형성 효과</t>
+          <t>MARVEL 초소형원자로에서 U–ZrH 및 MOX 핵연료봉의 정상운전 및 LOCA 성능에 대한 핵연료 형태의 영향</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -10480,7 +10480,7 @@
       </c>
       <c r="C100" s="9" t="inlineStr">
         <is>
-          <t>MHPR의 종횡비가 큰 고온 나트륨 히트 파이프의 성능 메커니즘 및 안정적인 작동 체제</t>
+          <t>MHPR용 대종횡비 고온 소듐 히트파이프의 성능 메커니즘 및 신뢰 운전 영역</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -10574,7 +10574,7 @@
       </c>
       <c r="C101" s="9" t="inlineStr">
         <is>
-          <t>주 펌프 상태 평가를 기반으로 한 SMR의 시스템 작동 제어 방법에 관한 연구</t>
+          <t>주냉각재펌프 건전성 평가 기반 SMR 계통 운전제어 방법 연구</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -10668,7 +10668,7 @@
       </c>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>이중 전도성 표면의 에폭시 패턴이 수영장 비등에 미치는 영향에 관한 실험적 연구</t>
+          <t>이중 전도성 표면의 에폭시 패턴이 풀비등에 미치는 영향에 관한 실험 연구</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="C103" s="9" t="inlineStr">
         <is>
-          <t>반사기의 분석 용액과 관련된 연료의 림프절 팽창 방법</t>
+          <t>반사체 해석해와 연계한 핵연료 영역 노달 전개법</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -10856,7 +10856,7 @@
       </c>
       <c r="C104" s="9" t="inlineStr">
         <is>
-          <t>An Agentic Multimodal RAG Framework for Enhancing Nuclear Regulatory Review: Preserving Structural Integrity of Safety Analysis Reports</t>
+          <t>원자력 규제심사 고도화를 위한 에이전트형 멀티모달 RAG 프레임워크: 안전성분석보고서의 구조적 무결성 보존</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="C105" s="9" t="inlineStr">
         <is>
-          <t>온도 구배에 의해 구동되는 이산화우라늄 내 기공 및 입자 경계의 이동: 위상 필드 시뮬레이션</t>
+          <t>온도구배에 의한 이산화우라늄 내 기공 및 결정립계 이동: 상장(phase-field) 모의</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11036,7 +11036,7 @@
       </c>
       <c r="C106" s="9" t="inlineStr">
         <is>
-          <t>고급 원자로를 위한 고장 안전 수동 안전 시스템의 PSA 정보에 입각한 설계 시사점</t>
+          <t>차세대 원자로의 고장 시 안전(fail-safe) 피동안전계통에 대한 PSA 정보 활용 설계 시사점</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -11130,7 +11130,7 @@
       </c>
       <c r="C107" s="9" t="inlineStr">
         <is>
-          <t>첨단 확산 및 분산 조건을 통해 상호 연결된 하위 채널에서 단상 및 2상 난류 혼합의 향상된 3D 모델링</t>
+          <t>고급 확산·분산항을 통한 상호연결 부수로 내 단상 및 2상 난류혼합의 향상된 3차원 모델링</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="C108" s="9" t="inlineStr">
         <is>
-          <t>PWR 연료봉 번들의 아냉각 비등에 대한 CRUD 침착 효과에 대한 수치 조사</t>
+          <t>PWR 핵연료봉 다발에서 CRUD 침적물이 과냉비등에 미치는 영향 수치해석</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -11310,7 +11310,7 @@
       </c>
       <c r="C109" s="9" t="inlineStr">
         <is>
-          <t>나선형 핵연료의 임계열유속 향상 보고에 관한 고찰: 비교 기준, 보정계수 일관성 및 룩업테이블 불확실성</t>
+          <t>나선형 핵연료의 임계열유속 향상 보고에 대한 고찰: 비교 기준, 보정계수 일관성 및 룩업테이블 불확실성</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -11404,7 +11404,7 @@
       </c>
       <c r="C110" s="9" t="inlineStr">
         <is>
-          <t>Eulerian 이상유동 접근법을 이용한 SIRIUS-3D 전규모 핵연료집합체 비등유동 시뮬레이션</t>
+          <t>오일러리안 2유체 접근법을 이용한 SIRIUS-3D 전체 핵연료집합체의 비등 유동 모의</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -11490,7 +11490,7 @@
       </c>
       <c r="C111" s="9" t="inlineStr">
         <is>
-          <t>SACCL: 방사선원 위치 추정을 위한 강화학습 기반 접근법</t>
+          <t>SACCL: 강화학습 기반 방사선원 위치 추정 기법</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="C112" s="9" t="inlineStr">
         <is>
-          <t>열시스템 안전 향상을 위한 비응축성 기체 존재하 복합 응축 열전달의 AI 기반 모델링</t>
+          <t>열계통 안전성 향상을 위한 비응축성 기체 존재 하 복합 응축 열전달의 AI 기반 모델링</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -11670,7 +11670,7 @@
       </c>
       <c r="C113" s="9" t="inlineStr">
         <is>
-          <t>수평 원형 가열관 내 헬륨-제논 혼합기체의 조성 성층화 특성 연구</t>
+          <t>수평 원형 가열관 내 헬륨-제논 혼합기체의 조성 성층 특성 연구</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -11764,7 +11764,7 @@
       </c>
       <c r="C114" s="9" t="inlineStr">
         <is>
-          <t>TMM과 MSM을 결합한 나선형 십자형 핵연료봉의 유동유발진동 응답</t>
+          <t>TMM과 MSM을 연계한 나선형 십자형 핵연료봉의 유동유발진동 응답</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -11858,7 +11858,7 @@
       </c>
       <c r="C115" s="9" t="inlineStr">
         <is>
-          <t>수직 해안 호안에서 쓰나미형 파랑 월파를 완화하기 위한 수중 수평판의 매개변수 평가</t>
+          <t>수직 호안에서 쓰나미성 파랑 월파 저감을 위한 수중 수평판의 매개변수 평가</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -11944,7 +11944,7 @@
       </c>
       <c r="C116" s="9" t="inlineStr">
         <is>
-          <t>납냉각 고속로 펌프의 신속한 유동장 복원을 위한 물리정보 기반 축소차수 모델링</t>
+          <t>납냉각 고속로 펌프 내 신속 유동장 재구성을 위한 물리정보 축소차수 모델링</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="C117" s="9" t="inlineStr">
         <is>
-          <t>동물 사체 폐기물 감용을 위한 통합 건조 및 다단 소각 공정의 개발과 평가: 방사성폐기물 관리에 대한 시사점</t>
+          <t>동물 사체 폐기물 감용을 위한 건조 및 다단 소각 통합 공정 개발 및 평가: 방사성폐기물 관리에 대한 시사점</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="C118" s="9" t="inlineStr">
         <is>
-          <t>서론: 원자력에 관한 사회기술적 연구—회고와 연구 분야 구축을 위한 의제</t>
+          <t>서론: 원자력 에너지의 사회기술적 연구 – 회고와 분야 구축을 위한 의제</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -12226,7 +12226,7 @@
       </c>
       <c r="C119" s="9" t="inlineStr">
         <is>
-          <t>적층제조 금속합금의 조사 영향: 최근 진전과 향후 전망</t>
+          <t>적층제조 금속 합금의 조사 효과: 최근 연구 동향 및 향후 전망</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -12414,7 +12414,7 @@
       </c>
       <c r="C121" s="9" t="inlineStr">
         <is>
-          <t>MSRE 디지털 트윈: 유한차분 모델링과 호스트 매개 듀얼 FPGA 실시간 에뮬레이션</t>
+          <t>MSRE 디지털트윈: 유한차분 모델링 및 호스트 매개 이중 FPGA 실시간 에뮬레이션</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="C122" s="9" t="inlineStr">
         <is>
-          <t>MTR 핵연료 설계에 토륨 도입이 미치는 영향—OSCAR-5를 이용한 SAFARI-1 평가</t>
+          <t>MTR 핵연료 설계에 토륨 도입의 영향 – OSCAR-5를 이용한 SAFARI-1 평가</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -12602,7 +12602,7 @@
       </c>
       <c r="C123" s="9" t="inlineStr">
         <is>
-          <t>저주파 중성자 잡음의 이해: KWU 원자로의 유동 이동 증거와 전역·국부 성분의 분리</t>
+          <t>저주파 중성자 잡음의 이해: KWU 원자로의 유동 편향 증거 및 전역·국부 성분 분리</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -12696,7 +12696,7 @@
       </c>
       <c r="C124" s="9" t="inlineStr">
         <is>
-          <t>축소차수 모델을 이용한 원전 열교환기의 과도 시뮬레이션</t>
+          <t>축소차수 모델을 이용한 원자력발전소 열교환기의 과도 모의</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -12790,7 +12790,7 @@
       </c>
       <c r="C125" s="9" t="inlineStr">
         <is>
-          <t>Korea-4GSR 사중극자석용 PCB 기반 버킹 회전코일 시스템 개발</t>
+          <t>Korea-4GSR 사중극 전자석용 PCB 기반 버킹 회전코일 시스템 개발</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -12884,7 +12884,7 @@
       </c>
       <c r="C126" s="9" t="inlineStr">
         <is>
-          <t>인공지능을 이용한 원전 사용후핵연료의 건식저장시설 이송 작업 예측</t>
+          <t>인공지능을 이용한 원자력발전소 사용후핵연료 요소의 건식저장 설비 이송 작업 예측</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -12978,7 +12978,7 @@
       </c>
       <c r="C127" s="9" t="inlineStr">
         <is>
-          <t>BN-600 원자로 저농축 구역의 Cr16-Ni19 오스테나이트강 핵연료 피복재에서 중성자 조사에 따른 변위 캐스케이드의 생성과 진화</t>
+          <t>BN-600 원자로 저농축 영역에서 중성자 조사 하 오스테나이트강 Cr16-Ni19 핵연료 피복관 내 변위 캐스케이드의 형성 및 전개</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="C128" s="9" t="inlineStr">
         <is>
-          <t>HTR-PM/Cu-Cl/ORC 열병합발전 시스템의 하이브리드 핀치해석 및 MLP 최적화</t>
+          <t>HTR-PM/Cu-Cl/ORC 열병합 시스템의 핀치 분석-MLP 하이브리드 최적화</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -13166,7 +13166,7 @@
       </c>
       <c r="C129" s="9" t="inlineStr">
         <is>
-          <t>3차원 비정렬 격자 중성자수송 문제를 위한 다단계 병렬 SN DFEM 알고리즘</t>
+          <t>3차원 비정렬 격자 중성자 수송 문제를 위한 다단계 병렬 SN DFEM 알고리즘</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -13260,7 +13260,7 @@
       </c>
       <c r="C130" s="9" t="inlineStr">
         <is>
-          <t>나선형 십자형 핵연료요소의 부식생성물 침적과 열전달 저하에 관한 수치 연구</t>
+          <t>나선형 십자형 핵연료 요소의 부식생성물 침적 및 열전달 열화 수치해석</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -13354,7 +13354,7 @@
       </c>
       <c r="C131" s="9" t="inlineStr">
         <is>
-          <t>원자력 해체 경로계획을 위한 RG-DRL</t>
+          <t>원자력시설 해체 경로계획을 위한 RG-DRL</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -13448,7 +13448,7 @@
       </c>
       <c r="C132" s="9" t="inlineStr">
         <is>
-          <t>단사정 지르코니아의 열전도도에 미치는 공공 결함의 영향: 분자동역학 시뮬레이션</t>
+          <t>공공 결함이 단사정 지르코니아 열전도도에 미치는 영향: 분자동역학 모의</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -13542,7 +13542,7 @@
       </c>
       <c r="C133" s="9" t="inlineStr">
         <is>
-          <t>납-비스무트 공융액 내 엇갈림형 나봉다발의 압력강하 기반 등가 횡류 저항 특성</t>
+          <t>납-비스무트 공정 내 엇갈림 배열 나봉 다발의 압력강하 기반 등가 횡류 저항 특성</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -13636,7 +13636,7 @@
       </c>
       <c r="C134" s="9" t="inlineStr">
         <is>
-          <t>액체납 히트파이프 냉각 마이크로리액터의 과도 열성능 및 안전성 평가</t>
+          <t>액체 납 히트파이프 냉각 초소형원자로의 과도 열성능 및 안전성 평가</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -13730,7 +13730,7 @@
       </c>
       <c r="C135" s="9" t="inlineStr">
         <is>
-          <t>VVER-1000 원자로 노심 냉각재 유동 및 열전달의 전산유체역학 시뮬레이션</t>
+          <t>VVER-1000 원자로 노심 내 냉각재 유동 및 열전달의 전산유체역학(CFD) 모의</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -13824,7 +13824,7 @@
       </c>
       <c r="C136" s="9" t="inlineStr">
         <is>
-          <t>몬테카를로 시뮬레이션을 이용한 고분자 재료의 브래그 피크 예측용 일반화 가능한 기계학습 프레임워크</t>
+          <t>몬테카를로 모의를 이용한 고분자 재료 내 브래그 피크 예측용 일반화 가능한 기계학습 프레임워크</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -13918,7 +13918,7 @@
       </c>
       <c r="C137" s="9" t="inlineStr">
         <is>
-          <t>GNP 강화 B4C-TiB2 복합재의 광자 차폐 응답: 실험 및 MCNP6.2 분석</t>
+          <t>GNP 강화 B4C-TiB2 복합재의 광자 차폐 특성: 실험 및 MCNP6.2 분석</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="C138" s="9" t="inlineStr">
         <is>
-          <t>파이로프로세싱-SFR 핵연료주기의 실물옵션 가치평가: 우라늄 가격 불확실성하 핵연료주기 비용의 의사결정 유연성 평가</t>
+          <t>파이로프로세싱-SFR 핵연료주기의 실물옵션 가치평가: 우라늄 가격 불확실성 하 핵연료주기 비용의 의사결정 유연성 평가</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -14106,7 +14106,7 @@
       </c>
       <c r="C139" s="9" t="inlineStr">
         <is>
-          <t>정오표: “독일 부지선정 절차—점토암 고준위방사성폐기물 처분장의 심도 한계에 관한 고찰”</t>
+          <t>정오표: 독일의 부지선정 절차: 점토암 내 고준위방사성폐기물 처분장의 심도 한계에 대한 고찰 [Prog. Nucl. Energy 201 (2026) 1-10 / 106555]</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -14200,7 +14200,7 @@
       </c>
       <c r="C140" s="9" t="inlineStr">
         <is>
-          <t>이중 경계 프레임워크가 열역학 평가에 미치는 영향: PWR 비교 엑서지 분석</t>
+          <t>이중 경계 프레임워크가 열역학 평가에 미치는 영향: PWR 엑서지 비교 분석</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="C141" s="9" t="inlineStr">
         <is>
-          <t>저주파 영역에서 원자로 노심 내부 핵연료집합체의 난류 유발 진동</t>
+          <t>저주파 영역에서 원자로 노심 내 핵연료집합체의 난류 유발 진동</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -14380,7 +14380,7 @@
       </c>
       <c r="C142" s="9" t="inlineStr">
         <is>
-          <t>ALWR 노심 부수로 특성 예측을 위한 Transformer 신경망과 고급 이상유동 상관식의 결합</t>
+          <t>트랜스포머 신경망과 고급 2상유동 상관식을 결합한 ALWR 노심 부수로 특성 예측</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -14474,7 +14474,7 @@
       </c>
       <c r="C143" s="9" t="inlineStr">
         <is>
-          <t>SCENES-CoreMelting의 용융물 재배치를 위한 결합 열전달 모델 개발 및 평가</t>
+          <t>SCENES-CoreMelting의 용융물 재배치를 위한 연계 열전달 모델 개발 및 평가</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -14568,7 +14568,7 @@
       </c>
       <c r="C144" s="9" t="inlineStr">
         <is>
-          <t>베이산 심지층 환경에서 테크네튬 화학종의 동적 거동과 변환: 고준위방사성폐기물 처분에 대한 시사점</t>
+          <t>베이산 심부 지질환경에서 테크네튬 화학종의 동적 거동 및 변환: 고준위방사성폐기물 처분에 대한 시사점</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="C145" s="9" t="inlineStr">
         <is>
-          <t>감마선 방출 패턴과 중성자 흡수단면적에 나타나는 핵 형상 공존의 관측 가능 특징</t>
+          <t>감마선 방출 패턴과 중성자 흡수 단면적에 나타나는 핵 형상 공존의 관측 가능한 징후</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -14756,7 +14756,7 @@
       </c>
       <c r="C146" s="9" t="inlineStr">
         <is>
-          <t>가속기구동 미임계시스템용 OpenMC의 실시간 다중 에너지영역 단면적 처리</t>
+          <t>가속기구동 미임계계통을 위한 OpenMC의 실시간 다중 에너지 영역 단면적 처리</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -14850,7 +14850,7 @@
       </c>
       <c r="C147" s="9" t="inlineStr">
         <is>
-          <t>사용후핵연료 운송사고 조건에서 UNet-Transformer 기반 방사성핵종 확산 예측</t>
+          <t>UNet-Transformer 기반 사용후핵연료 운반 사고 조건에서의 방사성핵종 확산 예측</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -14944,7 +14944,7 @@
       </c>
       <c r="C148" s="9" t="inlineStr">
         <is>
-          <t>불확실성을 고려한 LWR 원자로 기기의 다물리 연속 형상 최적화</t>
+          <t>불확실성 하 경수로 원자로 구성품의 다중물리 연속 형상 최적화</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -15038,7 +15038,7 @@
       </c>
       <c r="C149" s="9" t="inlineStr">
         <is>
-          <t>원전 비상운전절차 수행 복잡도 정량화를 위한 정보흐름 모델: 주과업과 부과업의 통합</t>
+          <t>원자력발전소 비상운전절차서 수행 복잡도 정량화를 위한 정보흐름 모델: 주업무 및 부업무 통합</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="C150" s="9" t="inlineStr">
         <is>
-          <t>이축 하중 조건에서 철근콘크리트 전단벽의 수치 연구</t>
+          <t>2축 하중 조건에서 철근콘크리트 전단벽의 수치해석 연구</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -15226,7 +15226,7 @@
       </c>
       <c r="C151" s="9" t="inlineStr">
         <is>
-          <t>PWR 격납건물 증기관 파단 열수력 CFD 모델링의 확인 및 검증(ATLAS-CUBE 벤치마크)</t>
+          <t>PWR 격납건물 내 증기배관 파단 열수력에 대한 CFD 모델링 검증 및 확인(ATLAS-CUBE 벤치마크)</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -15320,7 +15320,7 @@
       </c>
       <c r="C152" s="9" t="inlineStr">
         <is>
-          <t>세계적 수준의 시뮬레이션 소프트웨어 개발과 유지: RELAP5 사례 연구</t>
+          <t>세계 수준 모의 소프트웨어의 개발과 유지: RELAP5 사례 연구</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="C153" s="9" t="inlineStr">
         <is>
-          <t>열 및 방사선 노출하 중량 EAFS-지오폴리머 콘크리트의 성능: 실험 및 기계학습 연구</t>
+          <t>열 및 방사선 노출 하 중량 EAFS-지오폴리머 콘크리트의 성능: 실험 및 기계학습 연구</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -15508,7 +15508,7 @@
       </c>
       <c r="C154" s="9" t="inlineStr">
         <is>
-          <t>횡동요 조건에서 환형 핵연료 채널의 유량분배 특성에 관한 실험 연구</t>
+          <t>요동 운동 조건에서 환형 핵연료 유로 내 유량분배 특성에 관한 실험 연구</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -15602,7 +15602,7 @@
       </c>
       <c r="C155" s="9" t="inlineStr">
         <is>
-          <t>PecTAF: PWR 격납건물과 PCS 열교환기 연계 해석을 위한 3차원 열수력 해석 코드</t>
+          <t>PecTAF: PWR 격납건물 및 PCS 열교환기 연계 3차원 열수력 해석 코드</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="C156" s="9" t="inlineStr">
         <is>
-          <t>해양 횡동요 조건에서 납-비스무트 자연순환의 축척 방법</t>
+          <t>해양 요동 조건에서 납-비스무트 자연순환의 척도 방법</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -15790,7 +15790,7 @@
       </c>
       <c r="C157" s="9" t="inlineStr">
         <is>
-          <t>열적 비평형 다공매질 모델 기반 데브리 베드 재관수 거동 연구</t>
+          <t>열적 비평형 다공성매질 모델 기반 잔해층 재관수 거동 연구</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -15884,7 +15884,7 @@
       </c>
       <c r="C158" s="9" t="inlineStr">
         <is>
-          <t>페블베드 원자로 내 입상유동의 통계 분석</t>
+          <t>페블베드 원자로 내 입자 유동의 통계적 분석</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -15978,7 +15978,7 @@
       </c>
       <c r="C159" s="9" t="inlineStr">
         <is>
-          <t>원전 안전설계 및 해석용 SCENES 코드의 개발과 검증</t>
+          <t>원자력발전소 안전 설계 및 해석을 위한 SCENES 코드 개발 및 검증</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -16072,7 +16072,7 @@
       </c>
       <c r="C160" s="9" t="inlineStr">
         <is>
-          <t>지그재그 채널 내 초임계 이산화탄소의 유동 및 열전달 저하에 관한 실험·수치 연구</t>
+          <t>지그재그 유로 내 초임계 이산화탄소의 유동 및 열전달 열화에 관한 실험 및 수치해석 연구</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -16166,7 +16166,7 @@
       </c>
       <c r="C161" s="9" t="inlineStr">
         <is>
-          <t>히트파이프 원자로 및 브레이튼 사이클 기반 원전의 모델링과 제어전략</t>
+          <t>히트파이프 원자로 및 브레이튼 사이클 계통 기반 원자력발전소 모델링 및 제어 전략</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -16260,7 +16260,7 @@
       </c>
       <c r="C162" s="9" t="inlineStr">
         <is>
-          <t>고속스펙트럼 이중유체원자로의 반응도 제어전략에 대한 중성자학적 평가</t>
+          <t>고속 스펙트럼 이중유체원자로(DFR)의 반응도 제어 전략에 대한 중성자 해석 평가</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -16354,7 +16354,7 @@
       </c>
       <c r="C163" s="9" t="inlineStr">
         <is>
-          <t>히트파이프 냉각 원자로의 비응축성 기체를 고려한 가열부 열수력 특성 수치 연구</t>
+          <t>히트파이프 냉각 원자로에서 비응축성 기체를 고려한 가열 단위의 열수력 특성 수치해석</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -16448,7 +16448,7 @@
       </c>
       <c r="C164" s="9" t="inlineStr">
         <is>
-          <t>PRA, 규제 및 보호계통 위험 정량화: 위험정보·성능기반 감독을 위한 DES/MPP 개선</t>
+          <t>PRA, 규제 및 보호계통 리스크 정량화: 리스크 정보 활용·성능 기반 규제감독을 위한 DES/MPP 개선</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -16542,7 +16542,7 @@
       </c>
       <c r="C165" s="9" t="inlineStr">
         <is>
-          <t>공극 팽윤 예측 불확실성의 정량화: 원자로 안전여유를 위한 적합성 예측 프레임워크</t>
+          <t>공극 팽윤 예측의 불확실성 정량화: 원자로 안전여유도를 위한 등각 예측 프레임워크</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -16636,7 +16636,7 @@
       </c>
       <c r="C166" s="9" t="inlineStr">
         <is>
-          <t>몬테카를로 중성자수송의 기하학적 민감도 분석을 위한 확률론적 수반가중 표면적분</t>
+          <t>몬테카를로 중성자 수송의 기하학적 민감도 해석을 위한 확률론적 수반가중 표면적분</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -16730,7 +16730,7 @@
       </c>
       <c r="C167" s="9" t="inlineStr">
         <is>
-          <t>전자빔 용접 원자로압력용기강의 중성자 조사시험 설계</t>
+          <t>전자빔 용접 원자로압력용기강의 중성자 조사시험 계획 설계</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -16824,7 +16824,7 @@
       </c>
       <c r="C168" s="9" t="inlineStr">
         <is>
-          <t>고온·고압 조건에서 RPV 하부 관통 랜스 헤드의 밀봉 누설 및 예압에 대한 NRBO-XGBoost 기반 예측</t>
+          <t>고온·고압 조건에서 RPV 하부 관통 랜스 헤드의 밀봉 누설 및 예하중에 대한 NRBO-XGBoost 기반 예측</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -16918,7 +16918,7 @@
       </c>
       <c r="C169" s="9" t="inlineStr">
         <is>
-          <t>새로운 가중 시공간 크리깅 모델 기반 과도 에어로졸 농도 역산 방법</t>
+          <t>새로운 가중 시공간 크리깅 모델 기반 과도 에어로졸 농도 역추정 방법</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -17012,7 +17012,7 @@
       </c>
       <c r="C170" s="9" t="inlineStr">
         <is>
-          <t>Hong Ngu 퇴적물 시료의 방사선학적 특성: 통계분석 접근법</t>
+          <t>Hong Ngu 퇴적물 시료의 방사선학적 특성: 통계적 분석 접근</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -17200,7 +17200,7 @@
       </c>
       <c r="C172" s="9" t="inlineStr">
         <is>
-          <t>삼중수소 표준가스를 이용한 휴대용 공기 중 삼중수소 감시기의 저농도 직접 교정시스템 개발</t>
+          <t>삼중수소 표준가스를 이용한 휴대용 공기 중 삼중수소 감시기의 저농도 직접 교정 시스템 개발</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -17294,7 +17294,7 @@
       </c>
       <c r="C173" s="9" t="inlineStr">
         <is>
-          <t>일반형 용융염원자로의 비보호 유량상실사고에 관한 연구</t>
+          <t>일반 용융염원자로의 비보호 유량상실사고에 관하여</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -17380,7 +17380,7 @@
       </c>
       <c r="C174" s="9" t="inlineStr">
         <is>
-          <t>페블베드 모듈형 원자로의 TRISO 핵연료 연소 특성</t>
+          <t>페블베드 모듈형 원자로에서 TRISO 핵연료의 연소 특성 평가</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -17474,7 +17474,7 @@
       </c>
       <c r="C175" s="9" t="inlineStr">
         <is>
-          <t>화학형태와 방출경로를 고려한 가압경수로 탄소-14 설계 선원항</t>
+          <t>화학형태 및 방출경로를 고려한 가압경수로 탄소-14 설계 선원항</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -17568,7 +17568,7 @@
       </c>
       <c r="C176" s="9" t="inlineStr">
         <is>
-          <t>안전·보안 평가 통합을 통한 원자력시설 위험 거버넌스 개선: 전문가 관점</t>
+          <t>안전 및 보안 평가 통합을 통한 원자력시설 리스크 거버넌스 개선: 전문가 관점</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -17662,7 +17662,7 @@
       </c>
       <c r="C177" s="9" t="inlineStr">
         <is>
-          <t>인력 가용성을 가정한 비상조직 구조 사례를 포함한 다중호기 인간·조직 신뢰도 분석 방법</t>
+          <t>인력 가용성을 가정한 비상조직 구조 사례연구를 포함한 다수기 인간 및 조직 신뢰도 분석 방법</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -17756,7 +17756,7 @@
       </c>
       <c r="C178" s="9" t="inlineStr">
         <is>
-          <t>통합 BARGE 방법과 랫드 모델을 이용한 오염매체 내 코발트 생체접근성 및 생체이용률 비교 평가</t>
+          <t>통합 BARGE 방법 및 쥐 모델을 이용한 오염 매체로부터 코발트의 생체접근성 및 생체이용률 비교 평가</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -17850,7 +17850,7 @@
       </c>
       <c r="C179" s="9" t="inlineStr">
         <is>
-          <t>요르단 원자력발전의 대중 수용성: 제도 신뢰와 위험-편익 인식을 확장한 계획행동이론</t>
+          <t>요르단의 원자력 대중 수용성: 제도적 신뢰 및 위험-편익 인식을 통한 계획행동이론 확장</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -18038,7 +18038,7 @@
       </c>
       <c r="C181" s="9" t="inlineStr">
         <is>
-          <t>다단 초임계 CO2 브레이튼-유기 랭킨 복합사이클 개발을 통한 발전: 배치설계, 열성능 및 전역최적화</t>
+          <t>다단 초임계 이산화탄소 브레이튼 및 유기랭킨 복합 사이클 개발을 통한 발전: 배치 설계, 열성능 및 전역 최적화</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -18132,7 +18132,7 @@
       </c>
       <c r="C182" s="9" t="inlineStr">
         <is>
-          <t>원자로 운전 예측을 위한 물리정보 기반 합성데이터 활용</t>
+          <t>물리정보 합성 데이터를 활용한 원자로 운전 예측</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -18226,7 +18226,7 @@
       </c>
       <c r="C183" s="9" t="inlineStr">
         <is>
-          <t>증강 불변다양체 기반 연소도 계산의 축소차수 모델링</t>
+          <t>증강 불변다양체 기반 연소 계산의 축소차수 모델링</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -18320,7 +18320,7 @@
       </c>
       <c r="C184" s="9" t="inlineStr">
         <is>
-          <t>미확인 오염과 높은 배경에서도 강건한 이중표적 방사성핵종 정량화용 잡음제거 오토인코더</t>
+          <t>미지 오염 및 고배경에 강건한 이중 표적 방사성핵종 정량용 잡음제거 오토인코더</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -18414,7 +18414,7 @@
       </c>
       <c r="C185" s="9" t="inlineStr">
         <is>
-          <t>혁신형 원전을 위한 코드·표준 및 디지털 기술 활용 권고</t>
+          <t>코드·표준 및 디지털 기술 활용 - 혁신 원자력발전소를 위한 권고사항</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -18508,7 +18508,7 @@
       </c>
       <c r="C186" s="9" t="inlineStr">
         <is>
-          <t>전형적인 해양 병진운동 조건에서 핵연료집합체 내 납-비스무트 공융액의 유동 및 열전달 특성 수치 연구</t>
+          <t>대표적 해양 병진운동 조건에서 핵연료집합체 내 납-비스무트 공정의 유동 및 열전달 특성 수치해석 연구</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -18602,7 +18602,7 @@
       </c>
       <c r="C187" s="9" t="inlineStr">
         <is>
-          <t>노외검출기 기반 조화합성법의 핀별 출력 복원 적용</t>
+          <t>노외 검출기 기반 조화함수 합성법의 봉단위 출력 재구성 적용</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="C188" s="9" t="inlineStr">
         <is>
-          <t>연소도 측정을 위한 CiADS 기반 Np-237 핵변환 실험계획 설계 및 감마분광 시뮬레이션</t>
+          <t>CiADS 기반 237Np 핵변환 실험 방안 설계 및 연소도 측정을 위한 감마 분광 모의</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -18782,7 +18782,7 @@
       </c>
       <c r="C189" s="9" t="inlineStr">
         <is>
-          <t>액체연료 용융염원자로용 고정밀 3차원 수반 중성자수송 계산모듈 개발 및 검증</t>
+          <t>액체핵연료 용융염원자로를 위한 고충실도 3차원 수반 중성자 수송 계산 모듈 개발 및 검증</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -18876,7 +18876,7 @@
       </c>
       <c r="C190" s="9" t="inlineStr">
         <is>
-          <t>방사성요오드 화학종에 따른 선량 영향: CANDU 중대사고 사례 연구</t>
+          <t>방사성 요오드 화학종의 선량 영향: CANDU 중대사고 사례 연구</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -19044,7 +19044,7 @@
       </c>
       <c r="C192" s="9" t="inlineStr">
         <is>
-          <t>무작위 충전 페블베드 배열의 고정밀 유속측정 실험 및 시공간 유동 분석</t>
+          <t>무작위 충전 페블베드 배열에서의 고충실도 속도 측정 실험 및 시공간 유동 분석</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -19138,7 +19138,7 @@
       </c>
       <c r="C193" s="9" t="inlineStr">
         <is>
-          <t>예기치 않은 통신 과도 시 원자로 운전을 위한 상태추정 및 축소차수 물리 기반 모델예측제어</t>
+          <t>예기치 않은 통신 과도상태 시 원자로 운전을 위한 상태추정 및 축소차수 물리모델 기반 모델예측제어</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -19232,7 +19232,7 @@
       </c>
       <c r="C194" s="9" t="inlineStr">
         <is>
-          <t>증기상 요오드 식별 기능을 갖춘 정전집진 기반 방사성핵종 공기시료채취기</t>
+          <t>기체 요오드 판별 기능을 갖춘 정전 집진 기반 방사성핵종 공기 시료채취기</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -19326,7 +19326,7 @@
       </c>
       <c r="C195" s="9" t="inlineStr">
         <is>
-          <t>악티나이드 탄산염계 산성화 중 상안정성을 지배하는 임계 디부틸인산 농도와 오존분해에 의한 열화</t>
+          <t>악티늄 탄산염계 산성화 시 상 안정성을 지배하는 임계 인산디부틸 농도 및 오존분해에 의한 분해</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -19420,7 +19420,7 @@
       </c>
       <c r="C196" s="9" t="inlineStr">
         <is>
-          <t>소형모듈원자로 디지털 I&amp;C 계통의 STPA에 다양성 및 심층방어 분석 통합</t>
+          <t>소형모듈원자로 디지털 계측제어계통을 위한 STPA에 다양성 및 심층방어 분석 통합</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -19514,7 +19514,7 @@
       </c>
       <c r="C197" s="9" t="inlineStr">
         <is>
-          <t>iPWR형 원자로 비상계획구역 설정을 위한 확률론적 모델체인 방법론</t>
+          <t>iPWR형 원자로의 비상계획구역 설정을 위한 확률론적 모델 체인 방법론</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -19600,7 +19600,7 @@
       </c>
       <c r="C198" s="9" t="inlineStr">
         <is>
-          <t>선정된 타이타네이트 화합물의 방사선 차폐 성능: 실험 및 이론 연구</t>
+          <t>선정된 티탄산염 화합물의 방사선 차폐 성능: 실험 및 이론 연구</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -19694,7 +19694,7 @@
       </c>
       <c r="C199" s="9" t="inlineStr">
         <is>
-          <t>최적화된 자기산란 보정 수송보정법을 적용한 판형 원자로용 MC/MOC 2단계 방법 개발</t>
+          <t>최적화된 자기산란 보정 수송보정 방법을 적용한 판형 원자로용 MC/MOC 2단계 방법 개발</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -19780,7 +19780,7 @@
       </c>
       <c r="C200" s="9" t="inlineStr">
         <is>
-          <t>좁은 직사각형 채널 내 LBE 유동 및 열전달: 상관식 개발과 부수로 코드 구현</t>
+          <t>좁은 직사각형 유로 내 LBE 유동 및 열전달: 상관식 개발 및 부수로 코드 구현</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -19874,7 +19874,7 @@
       </c>
       <c r="C201" s="9" t="inlineStr">
         <is>
-          <t>일반형 iPWR 설계기준사고 시퀀스에 대한 MELCOR와 ASTEC 코드 간 비교</t>
+          <t>일반 iPWR의 설계기준사고 시퀀스에 대한 MELCOR와 ASTEC 코드 간 비교</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -19968,7 +19968,7 @@
       </c>
       <c r="C202" s="9" t="inlineStr">
         <is>
-          <t>토륨-우라늄 혼합 옥살레이트의 열분해 및 수열분해 비교: 상변화와 미세구조 특성</t>
+          <t>혼합 토륨–우라늄 옥살산염의 열분해 및 수열분해 비교: 상 변화 및 미세조직 특성</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -20054,7 +20054,7 @@
       </c>
       <c r="C203" s="9" t="inlineStr">
         <is>
-          <t>Zircaloy 피복재의 다중스케일 모델링: 기계론적 결정소성에서 시나리오 기반 검증을 갖춘 유한요소 대리모델까지</t>
+          <t>지르칼로이 피복관의 다중스케일 모델링: 메커니즘 기반 결정소성에서 유한요소 대리모델까지 및 시나리오 기반 검증</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -20148,7 +20148,7 @@
       </c>
       <c r="C204" s="9" t="inlineStr">
         <is>
-          <t>고온시험시설의 CATHARE3 모델 설명 및 HTGR 열수력 벤치마크 참여</t>
+          <t>고온시험시설(HTTF)의 CATHARE3 모델 기술 및 HTGR 열수력 벤치마크 참여</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -20336,7 +20336,7 @@
       </c>
       <c r="C206" s="9" t="inlineStr">
         <is>
-          <t>초임계 CO2 원심압축기 성능에 미치는 Xe 첨가의 영향</t>
+          <t>Xe 첨가가 초임계 CO2 원심압축기 성능에 미치는 영향</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -20430,7 +20430,7 @@
       </c>
       <c r="C207" s="9" t="inlineStr">
         <is>
-          <t>MAEO: 대규모 최적화 응용을 위한 확장 가능한 다목적 애니모픽 앙상블 최적화</t>
+          <t>MAEO: 대규모 최적화 응용을 위한 확장 가능한 다목적 Animorphic 앙상블 최적화</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -20524,7 +20524,7 @@
       </c>
       <c r="C208" s="9" t="inlineStr">
         <is>
-          <t>지하 화학폭발 후 터널 환기에 의한 가스 포집 평가</t>
+          <t>지하 화학 폭발 후 터널 환기를 통한 기체 포집 평가</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -20618,7 +20618,7 @@
       </c>
       <c r="C209" s="9" t="inlineStr">
         <is>
-          <t>ANSYS Fluent를 이용한 맥동 체판탑 수력학의 CFD 시뮬레이션: 통합 다상유동 모델링 접근법</t>
+          <t>ANSYS Fluent를 이용한 맥동 체판탑 내 유체역학의 CFD 모의: 통합 다상유동 모델링 접근</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -20712,7 +20712,7 @@
       </c>
       <c r="C210" s="9" t="inlineStr">
         <is>
-          <t>지수적으로 신장하는 표면 위 2차 나노유체 정체점 유동에 대한 줄가열 및 비선형 열복사의 복합 영향</t>
+          <t>지수적으로 늘어나는 표면 위 2차 나노유체 정체점 유동에 대한 줄 가열 및 비선형 열복사의 복합 영향</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -20900,7 +20900,7 @@
       </c>
       <c r="C212" s="9" t="inlineStr">
         <is>
-          <t>폐기물 인수기준하 실제 중준위 액체폐기물용 제올라이트 개질 시멘트 고화의 실용 검증</t>
+          <t>폐기물 인수기준(WAC)에 따른 실제 중준위 액체폐기물의 제올라이트 개질 시멘트 고화 실증 검증</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -20994,7 +20994,7 @@
       </c>
       <c r="C213" s="9" t="inlineStr">
         <is>
-          <t>온도별 석출강화 가공 FeCrAl 피복관의 열크리프 거동</t>
+          <t>석출강화 가공 FeCrAl 피복관의 온도별 열 크리프 거동</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -21088,7 +21088,7 @@
       </c>
       <c r="C214" s="9" t="inlineStr">
         <is>
-          <t>이종금속 용접부 응력부식균열 선단의 역학적 상태에 미치는 균열 위치의 영향</t>
+          <t>이종금속 용접부 응력부식균열 선단의 역학적 상태에 대한 균열 위치의 영향</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -21182,7 +21182,7 @@
       </c>
       <c r="C215" s="9" t="inlineStr">
         <is>
-          <t>NEMA NU 2-2007을 이용한 디지털 PET/CT 시스템의 정량적 벤치마킹 및 불확실성 기반 성능평가</t>
+          <t>NEMA NU 2–2007을 이용한 디지털 PET/CT 시스템의 정량적 벤치마킹 및 불확실성 기반 성능 평가</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -21276,7 +21276,7 @@
       </c>
       <c r="C216" s="9" t="inlineStr">
         <is>
-          <t>TRISO-ATOPS: 기체냉각로용 기계론적 선원항 모델</t>
+          <t>TRISO-ATOPS: 가스냉각로를 위한 메커니즘 기반 선원항 모델</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -21368,7 +21368,11 @@
           <t>Development of a multi-fluid and multi-condition heat transfer model for supercritical fluids based on incremental learning</t>
         </is>
       </c>
-      <c r="C217" s="9" t="inlineStr"/>
+      <c r="C217" s="9" t="inlineStr">
+        <is>
+          <t>증분학습 기반 초임계유체의 다유체·다조건 열전달 모델 개발</t>
+        </is>
+      </c>
       <c r="D217" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -21450,7 +21454,11 @@
           <t>Numerical investigation of coolant mixing and boron diffusion in PWR reactor pressure vessel using multi-scale coupling method</t>
         </is>
       </c>
-      <c r="C218" s="9" t="inlineStr"/>
+      <c r="C218" s="9" t="inlineStr">
+        <is>
+          <t>다중스케일 연계 방법을 이용한 PWR 원자로압력용기 내 냉각재 혼합 및 붕소 확산 수치해석</t>
+        </is>
+      </c>
       <c r="D218" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -21532,7 +21540,11 @@
           <t>Conceptual design of the ULGEN-150 space nuclear reactor core</t>
         </is>
       </c>
-      <c r="C219" s="9" t="inlineStr"/>
+      <c r="C219" s="9" t="inlineStr">
+        <is>
+          <t>ULGEN-150 우주용 원자로 노심 개념설계</t>
+        </is>
+      </c>
       <c r="D219" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -21614,7 +21626,11 @@
           <t>Experimental investigation and mechanism modeling of cold wall effect on critical heat flux in annular channels</t>
         </is>
       </c>
-      <c r="C220" s="9" t="inlineStr"/>
+      <c r="C220" s="9" t="inlineStr">
+        <is>
+          <t>환형 유로에서 냉벽 효과가 임계열유속에 미치는 영향의 실험 연구 및 메커니즘 모델링</t>
+        </is>
+      </c>
       <c r="D220" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -21696,7 +21712,11 @@
           <t>FROBA software update and its application in assessing the impact of Mo disks on UO2-Zr fuel rod performance</t>
         </is>
       </c>
-      <c r="C221" s="9" t="inlineStr"/>
+      <c r="C221" s="9" t="inlineStr">
+        <is>
+          <t>FROBA 소프트웨어 개선 및 Mo 디스크가 UO2-Zr 핵연료봉 성능에 미치는 영향 평가 적용</t>
+        </is>
+      </c>
       <c r="D221" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -21770,7 +21790,11 @@
           <t>Inspection of nuclear fuel rod surface defects under simulated underwater-like degradation</t>
         </is>
       </c>
-      <c r="C222" s="9" t="inlineStr"/>
+      <c r="C222" s="9" t="inlineStr">
+        <is>
+          <t>수중 모사 열화 조건에서의 핵연료봉 표면 결함 검사</t>
+        </is>
+      </c>
       <c r="D222" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -21852,7 +21876,11 @@
           <t>AP300 SMR: the design and its experimental basis</t>
         </is>
       </c>
-      <c r="C223" s="9" t="inlineStr"/>
+      <c r="C223" s="9" t="inlineStr">
+        <is>
+          <t>AP300 SMR: 설계 및 실험적 근거</t>
+        </is>
+      </c>
       <c r="D223" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -21934,7 +21962,11 @@
           <t>Rate-of-rise characterization of as-manufactured heat pipe mesh screen wick structures with an annular gap</t>
         </is>
       </c>
-      <c r="C224" s="9" t="inlineStr"/>
+      <c r="C224" s="9" t="inlineStr">
+        <is>
+          <t>환형 간극을 갖는 제작 상태 히트파이프 메시 스크린 윅 구조의 상승률 특성 평가</t>
+        </is>
+      </c>
       <c r="D224" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -22016,7 +22048,11 @@
           <t>Evaluation of aerial monitoring data by extended stripping window method</t>
         </is>
       </c>
-      <c r="C225" s="9" t="inlineStr"/>
+      <c r="C225" s="9" t="inlineStr">
+        <is>
+          <t>확장 스트리핑 윈도우 방법에 의한 항공 모니터링 데이터 평가</t>
+        </is>
+      </c>
       <c r="D225" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -22090,7 +22126,11 @@
           <t>Optimization of chemical etching conditions and evaluation of detection performance for the DX-22 solid-state nuclear track detector</t>
         </is>
       </c>
-      <c r="C226" s="9" t="inlineStr"/>
+      <c r="C226" s="9" t="inlineStr">
+        <is>
+          <t>DX-22 고체 비적 검출기의 화학 식각 조건 최적화 및 검출 성능 평가</t>
+        </is>
+      </c>
       <c r="D226" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -22172,7 +22212,11 @@
           <t>Corrosion and electrochemical response of 316L stainless steel in boron-free small modular reactor environments with KOH and NH3</t>
         </is>
       </c>
-      <c r="C227" s="9" t="inlineStr"/>
+      <c r="C227" s="9" t="inlineStr">
+        <is>
+          <t>KOH 및 NH3를 사용하는 무붕산 소형모듈원자로 환경에서 316L 스테인리스강의 부식 및 전기화학적 반응</t>
+        </is>
+      </c>
       <c r="D227" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -22254,7 +22298,11 @@
           <t>Neutronics analysis and design of mechanical shim control strategy for a pressurized water reactors under base load operation</t>
         </is>
       </c>
-      <c r="C228" s="9" t="inlineStr"/>
+      <c r="C228" s="9" t="inlineStr">
+        <is>
+          <t>기저부하 운전 가압경수로를 위한 기계적 심 제어 전략의 중성자 해석 및 설계</t>
+        </is>
+      </c>
       <c r="D228" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -22336,7 +22384,11 @@
           <t>Fast thermal-hydraulic-neutronic model to simulate transient behavior of an aqueous homogeneous reactor</t>
         </is>
       </c>
-      <c r="C229" s="9" t="inlineStr"/>
+      <c r="C229" s="9" t="inlineStr">
+        <is>
+          <t>수용액 균질로 과도 거동 모의를 위한 고속 열수력-중성자 연계 모델</t>
+        </is>
+      </c>
       <c r="D229" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -22418,7 +22470,11 @@
           <t>Global seismic site characterization of nuclear power plant sites using USGS Vs30 data</t>
         </is>
       </c>
-      <c r="C230" s="9" t="inlineStr"/>
+      <c r="C230" s="9" t="inlineStr">
+        <is>
+          <t>USGS Vs30 데이터를 이용한 원자력발전소 부지의 전 지구적 지진 부지 특성 평가</t>
+        </is>
+      </c>
       <c r="D230" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -22492,7 +22548,11 @@
           <t>Atmospheric Dispersion of Radioactive Materials Modeled by Stochastic Differential Equations</t>
         </is>
       </c>
-      <c r="C231" s="9" t="inlineStr"/>
+      <c r="C231" s="9" t="inlineStr">
+        <is>
+          <t>확률미분방정식으로 모델링한 방사성물질의 대기확산</t>
+        </is>
+      </c>
       <c r="D231" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -22574,7 +22634,11 @@
           <t>Development of a Modelica-based thermal-hydraulic code for an SCO2 Brayton cycle MMR and its application to accident analysis with PCHE</t>
         </is>
       </c>
-      <c r="C232" s="9" t="inlineStr"/>
+      <c r="C232" s="9" t="inlineStr">
+        <is>
+          <t>SCO2 브레이튼 사이클 MMR용 Modelica 기반 열수력 코드 개발 및 PCHE 사고해석 적용</t>
+        </is>
+      </c>
       <c r="D232" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -22656,7 +22720,11 @@
           <t>Numerical simulation of the solid-phase oxygen control mass exchanger in lead-bismuth fast reactors based on CFD-DEM coupling</t>
         </is>
       </c>
-      <c r="C233" s="9" t="inlineStr"/>
+      <c r="C233" s="9" t="inlineStr">
+        <is>
+          <t>CFD-DEM 연계 기반 납-비스무트 고속로 고상 산소제어 물질교환기의 수치 모의</t>
+        </is>
+      </c>
       <c r="D233" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -22738,7 +22806,11 @@
           <t>A Hybrid Fast Gauss Transform algorithm for Doppler Broadening of neutron cross section at extremely high temperatures</t>
         </is>
       </c>
-      <c r="C234" s="9" t="inlineStr"/>
+      <c r="C234" s="9" t="inlineStr">
+        <is>
+          <t>초고온에서 중성자 단면적 도플러 확장을 위한 하이브리드 고속 가우스 변환 알고리즘</t>
+        </is>
+      </c>
       <c r="D234" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -22820,7 +22892,11 @@
           <t>A neutron transport calculation method based on Monte Carlo–Deep learning–interface current coupling and its validation in assembly problems</t>
         </is>
       </c>
-      <c r="C235" s="9" t="inlineStr"/>
+      <c r="C235" s="9" t="inlineStr">
+        <is>
+          <t>몬테카를로–딥러닝–경계면 흐름 결합 기반 중성자 수송 계산 방법 및 집합체 문제 검증</t>
+        </is>
+      </c>
       <c r="D235" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -22902,7 +22978,11 @@
           <t>CFD–DEM investigation of drag mapping and discharge-rate effects in the HTR-10 moving pebble bed</t>
         </is>
       </c>
-      <c r="C236" s="9" t="inlineStr"/>
+      <c r="C236" s="9" t="inlineStr">
+        <is>
+          <t>HTR-10 이동 페블베드에서 항력 매핑 및 배출 속도 영향에 대한 CFD–DEM 연구</t>
+        </is>
+      </c>
       <c r="D236" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -22984,7 +23064,11 @@
           <t>Chaotic characteristics and state classification of pressure fluctuations in phase-change condensation water hammer</t>
         </is>
       </c>
-      <c r="C237" s="9" t="inlineStr"/>
+      <c r="C237" s="9" t="inlineStr">
+        <is>
+          <t>상변화 응축 수격현상에서 압력 변동의 혼돈 특성 및 상태 분류</t>
+        </is>
+      </c>
       <c r="D237" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -23066,7 +23150,11 @@
           <t>Cross-domain generalization for nuclear power plant classification using large language models</t>
         </is>
       </c>
-      <c r="C238" s="9" t="inlineStr"/>
+      <c r="C238" s="9" t="inlineStr">
+        <is>
+          <t>대규모 언어모델을 이용한 원자력발전소 분류의 교차 도메인 일반화</t>
+        </is>
+      </c>
       <c r="D238" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -23148,7 +23236,11 @@
           <t>Research on the efficient and lightweight surrogate model for Probabilistic Safety Margin analysis of SBLOCA in nuclear power plants integrating DL-TL</t>
         </is>
       </c>
-      <c r="C239" s="9" t="inlineStr"/>
+      <c r="C239" s="9" t="inlineStr">
+        <is>
+          <t>DL-TL을 통합한 원자력발전소 SBLOCA 확률론적 안전여유도 해석용 고효율 경량 대리모델 연구</t>
+        </is>
+      </c>
       <c r="D239" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -23230,7 +23322,11 @@
           <t>Validation and reliability analysis of CFD-based atmospheric dispersion modeling against wind tunnel experiments at a nuclear power plant site with irregular buildings and complex terrain</t>
         </is>
       </c>
-      <c r="C240" s="9" t="inlineStr"/>
+      <c r="C240" s="9" t="inlineStr">
+        <is>
+          <t>불규칙 건물 및 복잡 지형을 갖는 원자력발전소 부지에서 풍동실험 대비 CFD 기반 대기확산 모델링의 검증 및 신뢰성 분석</t>
+        </is>
+      </c>
       <c r="D240" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -23312,7 +23408,11 @@
           <t>Multiobjective optimization methodology for the design of a 10-kW-class space nuclear fission power system</t>
         </is>
       </c>
-      <c r="C241" s="9" t="inlineStr"/>
+      <c r="C241" s="9" t="inlineStr">
+        <is>
+          <t>10 kW급 우주 원자력 핵분열 전력계통 설계를 위한 다목적 최적화 방법론</t>
+        </is>
+      </c>
       <c r="D241" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -23394,7 +23494,11 @@
           <t>Seismic analysis of TMSR graphite core with viscous damping</t>
         </is>
       </c>
-      <c r="C242" s="9" t="inlineStr"/>
+      <c r="C242" s="9" t="inlineStr">
+        <is>
+          <t>점성감쇠를 고려한 TMSR 흑연 노심의 지진 해석</t>
+        </is>
+      </c>
       <c r="D242" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -23476,7 +23580,11 @@
           <t>Is grid-based intraoperative electron radiotherapy (IOERT) a potential solution for surface dose enhancement in breast cancer treatment?</t>
         </is>
       </c>
-      <c r="C243" s="9" t="inlineStr"/>
+      <c r="C243" s="9" t="inlineStr">
+        <is>
+          <t>격자 기반 수술 중 전자선 방사선치료(IOERT)는 유방암 치료에서 표면선량 증가를 위한 잠재적 해법인가?</t>
+        </is>
+      </c>
       <c r="D243" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -23550,7 +23658,11 @@
           <t>Optimization of a BWR bundle performance for reactor-grade plutonium and minor actinides recycling</t>
         </is>
       </c>
-      <c r="C244" s="9" t="inlineStr"/>
+      <c r="C244" s="9" t="inlineStr">
+        <is>
+          <t>원자로급 플루토늄 및 부악티늄 재활용을 위한 BWR 핵연료다발 성능 최적화</t>
+        </is>
+      </c>
       <c r="D244" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -23632,7 +23744,11 @@
           <t>Financing Nuclear Decommissioning in Ghana: An Evaluation of Public-Private Partnership Models</t>
         </is>
       </c>
-      <c r="C245" s="9" t="inlineStr"/>
+      <c r="C245" s="9" t="inlineStr">
+        <is>
+          <t>가나의 원자력시설 해체 재원 조달: 민관협력 모델 평가</t>
+        </is>
+      </c>
       <c r="D245" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -23714,7 +23830,11 @@
           <t>Divergent and moderating determinants of social and local acceptance of high-level radioactive waste facilities: The role of nuclear power risk perceptions</t>
         </is>
       </c>
-      <c r="C246" s="9" t="inlineStr"/>
+      <c r="C246" s="9" t="inlineStr">
+        <is>
+          <t>고준위방사성폐기물 시설의 사회적·지역적 수용성의 상이한 결정요인 및 조절요인: 원자력 위험인식의 역할</t>
+        </is>
+      </c>
       <c r="D246" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -23796,7 +23916,11 @@
           <t>Editorial Board</t>
         </is>
       </c>
-      <c r="C247" s="9" t="inlineStr"/>
+      <c r="C247" s="9" t="inlineStr">
+        <is>
+          <t>편집위원회</t>
+        </is>
+      </c>
       <c r="D247" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -23870,7 +23994,11 @@
           <t>Sensitivity analysis of fast neutron flux calculations for the RPV extended beltline region</t>
         </is>
       </c>
-      <c r="C248" s="9" t="inlineStr"/>
+      <c r="C248" s="9" t="inlineStr">
+        <is>
+          <t>원자로압력용기 확장 벨트라인 영역 고속중성자속 계산의 민감도 분석</t>
+        </is>
+      </c>
       <c r="D248" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -23952,7 +24080,11 @@
           <t>Site selection procedure in Germany: Considerations on a depth limit for a high-level radioactive waste repository in claystone</t>
         </is>
       </c>
-      <c r="C249" s="9" t="inlineStr"/>
+      <c r="C249" s="9" t="inlineStr">
+        <is>
+          <t>독일의 부지선정 절차: 점토암 내 고준위방사성폐기물 처분장의 심도 한계에 대한 고찰</t>
+        </is>
+      </c>
       <c r="D249" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -24034,7 +24166,11 @@
           <t>Analysis of the proliferation resistance of re-enriched reprocessed uranium on multiple recycling in nuclear reactors</t>
         </is>
       </c>
-      <c r="C250" s="9" t="inlineStr"/>
+      <c r="C250" s="9" t="inlineStr">
+        <is>
+          <t>원자로 내 다중 재활용 시 재농축 재처리우라늄의 핵확산저항성 분석</t>
+        </is>
+      </c>
       <c r="D250" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -24108,7 +24244,11 @@
           <t>Central-Difference method based on consistent Half-Node linear approximation for the neutron diffusion equation</t>
         </is>
       </c>
-      <c r="C251" s="9" t="inlineStr"/>
+      <c r="C251" s="9" t="inlineStr">
+        <is>
+          <t>중성자 확산방정식을 위한 일관된 반노드 선형근사 기반 중심차분법</t>
+        </is>
+      </c>
       <c r="D251" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -24190,7 +24330,11 @@
           <t>Design and analysis of secondary-side passive residual heat removal system to enhance inherent safety of lead-bismuth fast reactor STELLAR-EX</t>
         </is>
       </c>
-      <c r="C252" s="9" t="inlineStr"/>
+      <c r="C252" s="9" t="inlineStr">
+        <is>
+          <t>납-비스무트 고속로 STELLAR-EX의 고유안전성 향상을 위한 2차측 피동잔열제거계통 설계 및 해석</t>
+        </is>
+      </c>
       <c r="D252" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -24264,7 +24408,11 @@
           <t>Development of a benchmark experimental method for large angle scattering cross section of 14 MeV neutrons using compound targets – Application to fluorine benchmarking using PTFE</t>
         </is>
       </c>
-      <c r="C253" s="9" t="inlineStr"/>
+      <c r="C253" s="9" t="inlineStr">
+        <is>
+          <t>복합 표적을 이용한 14 MeV 중성자 대각도 산란 단면적 벤치마크 실험법 개발 – PTFE를 이용한 불소 벤치마킹 적용</t>
+        </is>
+      </c>
       <c r="D253" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -24338,7 +24486,11 @@
           <t>Effect of burnup-dependent gap conductance on fuel–clad mechanical interaction and PCI risk during transient power excursions</t>
         </is>
       </c>
-      <c r="C254" s="9" t="inlineStr"/>
+      <c r="C254" s="9" t="inlineStr">
+        <is>
+          <t>과도 출력 급상승 시 연소도 의존 간극 열전도도가 핵연료-피복관 기계적 상호작용 및 PCI 위험에 미치는 영향</t>
+        </is>
+      </c>
       <c r="D254" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -24412,7 +24564,11 @@
           <t>Multiresolution Photon Dose Reconstruction using FLUKA and Resolution-Adaptive Physics-Informed Neural Networks</t>
         </is>
       </c>
-      <c r="C255" s="9" t="inlineStr"/>
+      <c r="C255" s="9" t="inlineStr">
+        <is>
+          <t>FLUKA와 해상도 적응형 물리정보신경망을 이용한 다중해상도 광자 선량 재구성</t>
+        </is>
+      </c>
       <c r="D255" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -24486,7 +24642,11 @@
           <t>Numerical investigation on flow instability in casing once-through steam generators based on subchannel method</t>
         </is>
       </c>
-      <c r="C256" s="9" t="inlineStr"/>
+      <c r="C256" s="9" t="inlineStr">
+        <is>
+          <t>부수로 방법 기반 케이싱형 관류식 증기발생기의 유동 불안정성 수치해석 연구</t>
+        </is>
+      </c>
       <c r="D256" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -24568,7 +24728,11 @@
           <t>Seismic fragility analysis of multi-line transmission structure based on gas-insulated switchgear (GIS) equipment for nuclear power applications</t>
         </is>
       </c>
-      <c r="C257" s="9" t="inlineStr"/>
+      <c r="C257" s="9" t="inlineStr">
+        <is>
+          <t>원자력 적용을 위한 가스절연개폐장치(GIS) 기반 다회선 송전구조물의 지진 취약도 해석</t>
+        </is>
+      </c>
       <c r="D257" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -24650,7 +24814,11 @@
           <t>CFD analysis of thermal mixing and stratification phenomena in a tee with a blind-end branch using URANS approach</t>
         </is>
       </c>
-      <c r="C258" s="9" t="inlineStr"/>
+      <c r="C258" s="9" t="inlineStr">
+        <is>
+          <t>URANS 접근법을 이용한 막힌 분기관 T자관의 열혼합 및 성층화 현상 CFD 해석</t>
+        </is>
+      </c>
       <c r="D258" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -24724,7 +24892,11 @@
           <t>Direct numerical simulation of thermal mixing in a T-junction with conjugate heat transfer in the solid walls</t>
         </is>
       </c>
-      <c r="C259" s="9" t="inlineStr"/>
+      <c r="C259" s="9" t="inlineStr">
+        <is>
+          <t>고체 벽 공액열전달을 고려한 T자 접합부 열혼합의 직접수치모사</t>
+        </is>
+      </c>
       <c r="D259" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -24806,7 +24978,11 @@
           <t>Modeling and decoupler design for the OTSG feedwater control system of small modular reactors</t>
         </is>
       </c>
-      <c r="C260" s="9" t="inlineStr"/>
+      <c r="C260" s="9" t="inlineStr">
+        <is>
+          <t>소형모듈원자로 OTSG 급수제어계통의 모델링 및 비연성화기 설계</t>
+        </is>
+      </c>
       <c r="D260" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -24880,7 +25056,11 @@
           <t>Properties of single-mode optical fibers under high-dose gamma-ray irradiation</t>
         </is>
       </c>
-      <c r="C261" s="9" t="inlineStr"/>
+      <c r="C261" s="9" t="inlineStr">
+        <is>
+          <t>고선량 감마선 조사 하 단일모드 광섬유의 특성</t>
+        </is>
+      </c>
       <c r="D261" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -24954,7 +25134,11 @@
           <t>Uncertainty analysis for nuclear design parameters of VHTR-350</t>
         </is>
       </c>
-      <c r="C262" s="9" t="inlineStr"/>
+      <c r="C262" s="9" t="inlineStr">
+        <is>
+          <t>VHTR-350 핵설계 변수의 불확실성 분석</t>
+        </is>
+      </c>
       <c r="D262" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -25028,7 +25212,11 @@
           <t>Application of artificial neural networks in the identification of nuclear power plant accident and transient</t>
         </is>
       </c>
-      <c r="C263" s="9" t="inlineStr"/>
+      <c r="C263" s="9" t="inlineStr">
+        <is>
+          <t>원자력발전소 사고 및 과도상태 식별에 대한 인공신경망 적용</t>
+        </is>
+      </c>
       <c r="D263" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -25102,7 +25290,11 @@
           <t>A parametric review of saturated pool boiling heat transfer over vertical tubes and tube bundles for passive residual heat removal systems</t>
         </is>
       </c>
-      <c r="C264" s="9" t="inlineStr"/>
+      <c r="C264" s="9" t="inlineStr">
+        <is>
+          <t>피동잔열제거계통을 위한 수직관 및 관다발 포화 풀비등 열전달의 매개변수별 고찰</t>
+        </is>
+      </c>
       <c r="D264" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -25184,7 +25376,11 @@
           <t>Method research on the neutronic simulations of the bowed fuel rods in nuclear reactors</t>
         </is>
       </c>
-      <c r="C265" s="9" t="inlineStr"/>
+      <c r="C265" s="9" t="inlineStr">
+        <is>
+          <t>원자로 내 휜 핵연료봉의 중성자 해석 모의 방법 연구</t>
+        </is>
+      </c>
       <c r="D265" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -25258,7 +25454,11 @@
           <t>Nuclide number density prediction in molten salt reactors using dynamic mode decomposition with fractional-power snapshot transformation</t>
         </is>
       </c>
-      <c r="C266" s="9" t="inlineStr"/>
+      <c r="C266" s="9" t="inlineStr">
+        <is>
+          <t>분수 거듭제곱 스냅샷 변환을 적용한 동적 모드 분해를 이용한 용융염원자로 핵종 수밀도 예측</t>
+        </is>
+      </c>
       <c r="D266" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -25340,7 +25540,11 @@
           <t>Numerical investigation of the effects of various non-condensable gases on steam condensation outside a vertical tube</t>
         </is>
       </c>
-      <c r="C267" s="9" t="inlineStr"/>
+      <c r="C267" s="9" t="inlineStr">
+        <is>
+          <t>다양한 비응축성 기체가 수직관 외부 증기 응축에 미치는 영향 수치해석 연구</t>
+        </is>
+      </c>
       <c r="D267" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -25414,7 +25618,11 @@
           <t>Acquisition-specific motion deblurring in X-ray radiography using a dual-acquisition residual-domain framework</t>
         </is>
       </c>
-      <c r="C268" s="9" t="inlineStr"/>
+      <c r="C268" s="9" t="inlineStr">
+        <is>
+          <t>이중 획득 잔차 영역 프레임워크를 이용한 X선 투과영상의 획득 특화 동작 흐림 제거</t>
+        </is>
+      </c>
       <c r="D268" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -25496,7 +25704,11 @@
           <t>Corrosion behavior of 304 stainless steel in pressurized water reactor primary water chemistry controlled by LiOH and KOH</t>
         </is>
       </c>
-      <c r="C269" s="9" t="inlineStr"/>
+      <c r="C269" s="9" t="inlineStr">
+        <is>
+          <t>LiOH 및 KOH로 제어된 가압경수로 1차계통 수화학 환경에서 304 스테인리스강의 부식 거동</t>
+        </is>
+      </c>
       <c r="D269" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -25570,7 +25782,11 @@
           <t>Diffusion of tritium in Li4SiO4 crystal: A first-principles study</t>
         </is>
       </c>
-      <c r="C270" s="9" t="inlineStr"/>
+      <c r="C270" s="9" t="inlineStr">
+        <is>
+          <t>Li4SiO4 결정 내 삼중수소 확산: 제1원리 연구</t>
+        </is>
+      </c>
       <c r="D270" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -25652,7 +25868,11 @@
           <t>Full-scale vibration fatigue testing of 316L butt-welded small-bore piping in nuclear power plants and equivalent structural stress S-N curve</t>
         </is>
       </c>
-      <c r="C271" s="9" t="inlineStr"/>
+      <c r="C271" s="9" t="inlineStr">
+        <is>
+          <t>원자력발전소 316L 맞대기 용접 소구경 배관의 실규모 진동 피로시험 및 등가구조응력 S-N 곡선</t>
+        </is>
+      </c>
       <c r="D271" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -25734,7 +25954,11 @@
           <t>Neutronic and depletion analysis of a 5 MWth heat pipe cooled reactor with TRISO fuel and fluoride salt using MCS</t>
         </is>
       </c>
-      <c r="C272" s="9" t="inlineStr"/>
+      <c r="C272" s="9" t="inlineStr">
+        <is>
+          <t>MCS를 이용한 TRISO 핵연료 및 불화염 적용 5 MWth 히트파이프 냉각 원자로의 중성자 및 연소 해석</t>
+        </is>
+      </c>
       <c r="D272" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -25816,7 +26040,11 @@
           <t>Vacuum leak detection and localization based on remote handling and laser spectroscopy coupling</t>
         </is>
       </c>
-      <c r="C273" s="9" t="inlineStr"/>
+      <c r="C273" s="9" t="inlineStr">
+        <is>
+          <t>원격취급과 레이저 분광 결합 기반 진공 누설 탐지 및 위치 추정</t>
+        </is>
+      </c>
       <c r="D273" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -25898,7 +26126,11 @@
           <t>Stabilization of Research Reactor Spent Nuclear Fuels: Pellet Formation Using Spark Plasma Sintering</t>
         </is>
       </c>
-      <c r="C274" s="9" t="inlineStr"/>
+      <c r="C274" s="9" t="inlineStr">
+        <is>
+          <t>연구로 사용후핵연료의 안정화: 방전플라즈마소결을 이용한 소결체 성형</t>
+        </is>
+      </c>
       <c r="D274" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -25980,7 +26212,11 @@
           <t>Thermal Aging Analysis of RNS-NR Neutron-Shielding Material for Long-Term Storage of Spent Nuclear Fuel</t>
         </is>
       </c>
-      <c r="C275" s="9" t="inlineStr"/>
+      <c r="C275" s="9" t="inlineStr">
+        <is>
+          <t>사용후핵연료 장기저장용 RNS-NR 중성자 차폐재의 열적 노화 분석</t>
+        </is>
+      </c>
       <c r="D275" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -26062,7 +26298,11 @@
           <t>A framework for probabilistic risk assessment of nuclear power plants coupled with data centers using causal analysis</t>
         </is>
       </c>
-      <c r="C276" s="9" t="inlineStr"/>
+      <c r="C276" s="9" t="inlineStr">
+        <is>
+          <t>인과분석을 이용한 데이터센터 연계 원자력발전소의 확률론적 리스크 평가 프레임워크</t>
+        </is>
+      </c>
       <c r="D276" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -26144,7 +26384,11 @@
           <t>Corrosion and mitigation of structural materials in chloride-based molten salt reactors: Mechanisms, challenges, and design strategies</t>
         </is>
       </c>
-      <c r="C277" s="9" t="inlineStr"/>
+      <c r="C277" s="9" t="inlineStr">
+        <is>
+          <t>염화물계 용융염원자로 구조재료의 부식 및 완화: 메커니즘, 과제 및 설계 전략</t>
+        </is>
+      </c>
       <c r="D277" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -26218,7 +26462,11 @@
           <t>Integration of PID controller and reinforcement learning agents for core power control of small pressurized water reactors</t>
         </is>
       </c>
-      <c r="C278" s="9" t="inlineStr"/>
+      <c r="C278" s="9" t="inlineStr">
+        <is>
+          <t>소형 가압경수로 노심출력 제어를 위한 PID 제어기와 강화학습 에이전트의 통합</t>
+        </is>
+      </c>
       <c r="D278" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -26292,7 +26540,11 @@
           <t>Precise location of failed fuel assembly in operating PWR-core based on fine nuclide evolution and deep metric learning</t>
         </is>
       </c>
-      <c r="C279" s="9" t="inlineStr"/>
+      <c r="C279" s="9" t="inlineStr">
+        <is>
+          <t>정밀 핵종 변화 및 심층 거리학습 기반 운전 중 PWR 노심 결함 핵연료집합체 위치 정밀 탐지</t>
+        </is>
+      </c>
       <c r="D279" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -26374,7 +26626,11 @@
           <t>Strategies for re-enriching depleted uranium: Reducing the consumption of natural UF6 for fuel production in a nuclear power reactor</t>
         </is>
       </c>
-      <c r="C280" s="9" t="inlineStr"/>
+      <c r="C280" s="9" t="inlineStr">
+        <is>
+          <t>감손우라늄 재농축 전략: 원자력발전로 핵연료 생산을 위한 천연 UF6 소비 저감</t>
+        </is>
+      </c>
       <c r="D280" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -26456,7 +26712,11 @@
           <t>Heterogeneity in community acceptance of urban SMR siting: A contingent valuation and latent class analysis</t>
         </is>
       </c>
-      <c r="C281" s="9" t="inlineStr"/>
+      <c r="C281" s="9" t="inlineStr">
+        <is>
+          <t>도심 SMR 부지선정에 대한 지역사회 수용성의 이질성: 조건부가치평가 및 잠재계층 분석</t>
+        </is>
+      </c>
       <c r="D281" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -26530,7 +26790,11 @@
           <t>Multi-objective optimization and thermodynamic limits of free-piston Stirling generators using physics-informed active learning</t>
         </is>
       </c>
-      <c r="C282" s="9" t="inlineStr"/>
+      <c r="C282" s="9" t="inlineStr">
+        <is>
+          <t>물리정보 능동학습을 이용한 자유피스톤 스털링 발전기의 다목적 최적화 및 열역학적 한계</t>
+        </is>
+      </c>
       <c r="D282" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -26604,7 +26868,11 @@
           <t>Coupled comparative simulation and comprehensive performance evaluation of steam-extraction schemes for CHP retrofit of HPR1000 nuclear power units</t>
         </is>
       </c>
-      <c r="C283" s="9" t="inlineStr"/>
+      <c r="C283" s="9" t="inlineStr">
+        <is>
+          <t>HPR1000 원자력발전소 열병합(CHP) 개조를 위한 증기 추기 방식의 연계 비교 모의 및 종합 성능 평가</t>
+        </is>
+      </c>
       <c r="D283" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -26686,7 +26954,11 @@
           <t>Diffusion-based phase space nodal method (PSN): Solving the neutron transport equation with a diffusion code</t>
         </is>
       </c>
-      <c r="C284" s="9" t="inlineStr"/>
+      <c r="C284" s="9" t="inlineStr">
+        <is>
+          <t>확산 기반 위상공간 노달 방법(PSN): 확산 코드를 이용한 중성자 수송방정식 풀이</t>
+        </is>
+      </c>
       <c r="D284" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -26768,7 +27040,11 @@
           <t>Numerical study of a guide shell for enhancing steam–air condensation heat transfer outside a straight tube</t>
         </is>
       </c>
-      <c r="C285" s="9" t="inlineStr"/>
+      <c r="C285" s="9" t="inlineStr">
+        <is>
+          <t>직관 외부 증기-공기 응축 열전달 향상을 위한 가이드 쉘의 수치해석 연구</t>
+        </is>
+      </c>
       <c r="D285" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -26850,7 +27126,11 @@
           <t>Study on vibration reduction mechanism of steam generator tube stabilizers based on damping control</t>
         </is>
       </c>
-      <c r="C286" s="9" t="inlineStr"/>
+      <c r="C286" s="9" t="inlineStr">
+        <is>
+          <t>감쇠 제어 기반 증기발생기 전열관 안정화기의 진동 저감 메커니즘 연구</t>
+        </is>
+      </c>
       <c r="D286" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -26932,7 +27212,11 @@
           <t>Analysis of dynamics of fuel rods in pulsed fast reactor</t>
         </is>
       </c>
-      <c r="C287" s="9" t="inlineStr"/>
+      <c r="C287" s="9" t="inlineStr">
+        <is>
+          <t>펄스형 고속로 핵연료봉의 동특성 해석</t>
+        </is>
+      </c>
       <c r="D287" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -27006,7 +27290,11 @@
           <t>Fragility analysis of PCCV under internal pressure via probability density evolution method</t>
         </is>
       </c>
-      <c r="C288" s="9" t="inlineStr"/>
+      <c r="C288" s="9" t="inlineStr">
+        <is>
+          <t>확률밀도진화법을 이용한 내압 하 PCCV의 취약도 해석</t>
+        </is>
+      </c>
       <c r="D288" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -27080,7 +27368,11 @@
           <t>Tailored potassium-alumino-borosilicate glasses for high-level immobilization of Cs+, Co2+, and Ni2+: Enhancing structural integrity, thermal and mechanical stability, and leaching resistance</t>
         </is>
       </c>
-      <c r="C289" s="9" t="inlineStr"/>
+      <c r="C289" s="9" t="inlineStr">
+        <is>
+          <t>Cs+, Co2+ 및 Ni2+의 고함량 고정화를 위한 맞춤형 칼륨-알루미노-붕규산염 유리: 구조적 건전성, 열적·기계적 안정성 및 침출 저항성 향상</t>
+        </is>
+      </c>
       <c r="D289" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -27162,7 +27454,11 @@
           <t>Effect of different oxidation time on deuterium absorption behavior of titanium films for radiation-voltaic isotope batteries</t>
         </is>
       </c>
-      <c r="C290" s="9" t="inlineStr"/>
+      <c r="C290" s="9" t="inlineStr">
+        <is>
+          <t>방사선-전지형 동위원소 전지용 티타늄 박막의 산화시간에 따른 중수소 흡수 거동</t>
+        </is>
+      </c>
       <c r="D290" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -27244,7 +27540,11 @@
           <t>Geometry optimization and fuel failure analysis for micro-scale PeLUIt-10 reactor</t>
         </is>
       </c>
-      <c r="C291" s="9" t="inlineStr"/>
+      <c r="C291" s="9" t="inlineStr">
+        <is>
+          <t>초소형 PeLUIt-10 원자로의 형상 최적화 및 핵연료 파손 해석</t>
+        </is>
+      </c>
       <c r="D291" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -27326,7 +27626,11 @@
           <t>Ml-based fission cross section calculations for 235,236,238U</t>
         </is>
       </c>
-      <c r="C292" s="9" t="inlineStr"/>
+      <c r="C292" s="9" t="inlineStr">
+        <is>
+          <t>ML 기반 235,236,238U 핵분열 단면적 계산</t>
+        </is>
+      </c>
       <c r="D292" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -27408,7 +27712,11 @@
           <t>Neutronic analysis of a two-region damaged reactor model based on the external source mode of the Serpent code</t>
         </is>
       </c>
-      <c r="C293" s="9" t="inlineStr"/>
+      <c r="C293" s="9" t="inlineStr">
+        <is>
+          <t>Serpent 코드 외부선원 모드 기반 2영역 손상 원자로 모델의 중성자 해석</t>
+        </is>
+      </c>
       <c r="D293" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -27490,7 +27798,11 @@
           <t>Rapid prediction of atmospheric radionuclide concentration at an AP1000 nuclear power plant with complex terrain using a neural network optimized by a quantum virus optimization algorithm</t>
         </is>
       </c>
-      <c r="C294" s="9" t="inlineStr"/>
+      <c r="C294" s="9" t="inlineStr">
+        <is>
+          <t>양자 바이러스 최적화 알고리즘으로 최적화한 신경망을 이용한 복잡 지형 AP1000 원자력발전소의 대기 중 방사성핵종 농도 신속 예측</t>
+        </is>
+      </c>
       <c r="D294" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -27572,7 +27884,11 @@
           <t>Study on the simultaneous impact of double droplets on a wetted cylindrical wall by the CLSVOF method</t>
         </is>
       </c>
-      <c r="C295" s="9" t="inlineStr"/>
+      <c r="C295" s="9" t="inlineStr">
+        <is>
+          <t>CLSVOF 방법을 이용한 젖은 원통 벽면에 대한 이중 액적 동시 충돌 연구</t>
+        </is>
+      </c>
       <c r="D295" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -27654,7 +27970,11 @@
           <t>Tungsten-based polymer composites for lead-free gamma-ray shielding: attenuation performance and mechanical trade-offs</t>
         </is>
       </c>
-      <c r="C296" s="9" t="inlineStr"/>
+      <c r="C296" s="9" t="inlineStr">
+        <is>
+          <t>무연 감마선 차폐용 텅스텐 기반 고분자 복합재: 감쇠 성능과 기계적 특성의 상충관계</t>
+        </is>
+      </c>
       <c r="D296" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -27736,7 +28056,11 @@
           <t>Analytical investigations on dynamic instabilities in large PHWRs</t>
         </is>
       </c>
-      <c r="C297" s="9" t="inlineStr"/>
+      <c r="C297" s="9" t="inlineStr">
+        <is>
+          <t>대형 PHWR의 동적 불안정성에 대한 해석적 연구</t>
+        </is>
+      </c>
       <c r="D297" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -27818,7 +28142,11 @@
           <t>Effect of leakage cavity geometry on the performance of a rim-driven high-load helium compressor</t>
         </is>
       </c>
-      <c r="C298" s="9" t="inlineStr"/>
+      <c r="C298" s="9" t="inlineStr">
+        <is>
+          <t>누설 공동 형상이 림구동 고부하 헬륨 압축기 성능에 미치는 영향</t>
+        </is>
+      </c>
       <c r="D298" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -27892,7 +28220,11 @@
           <t>Supervisory Control of Nuclear Power Plants Using Finite State Automata</t>
         </is>
       </c>
-      <c r="C299" s="9" t="inlineStr"/>
+      <c r="C299" s="9" t="inlineStr">
+        <is>
+          <t>유한상태 오토마타를 이용한 원자력발전소 감시제어</t>
+        </is>
+      </c>
       <c r="D299" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -27974,7 +28306,11 @@
           <t>Acceleration methods for the preprocessing of three-dimensional discrete ordinates radiation shielding calculations</t>
         </is>
       </c>
-      <c r="C300" s="9" t="inlineStr"/>
+      <c r="C300" s="9" t="inlineStr">
+        <is>
+          <t>3차원 이산좌표 방사선 차폐 계산 전처리 가속 기법</t>
+        </is>
+      </c>
       <c r="D300" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -28056,7 +28392,11 @@
           <t>Analysis of severe accident progression in a BWR considering power uprates and ATF cladding materials</t>
         </is>
       </c>
-      <c r="C301" s="9" t="inlineStr"/>
+      <c r="C301" s="9" t="inlineStr">
+        <is>
+          <t>출력증강 및 ATF 피복관 재료를 고려한 BWR 중대사고 진행 해석</t>
+        </is>
+      </c>
       <c r="D301" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -28138,7 +28478,11 @@
           <t>Direct incorporation of up-scattering sources in the Resonance Spectrum Expansion (RSE) method</t>
         </is>
       </c>
-      <c r="C302" s="9" t="inlineStr"/>
+      <c r="C302" s="9" t="inlineStr">
+        <is>
+          <t>공명 스펙트럼 전개(RSE) 방법에서의 상향산란 선원 직접 반영</t>
+        </is>
+      </c>
       <c r="D302" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -28220,7 +28564,11 @@
           <t>Hybrid deep learning and metaheuristic algorithms for contaminated zone prediction and source term inversion in nuclear safety</t>
         </is>
       </c>
-      <c r="C303" s="9" t="inlineStr"/>
+      <c r="C303" s="9" t="inlineStr">
+        <is>
+          <t>원자력 안전에서의 오염구역 예측 및 선원항 역산을 위한 하이브리드 딥러닝·메타휴리스틱 알고리즘</t>
+        </is>
+      </c>
       <c r="D303" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -28302,7 +28650,11 @@
           <t>Neutronic analysis of Yttrium Hydride temperature feedback coefficient in HALEU UMo fuelled microreactors</t>
         </is>
       </c>
-      <c r="C304" s="9" t="inlineStr"/>
+      <c r="C304" s="9" t="inlineStr">
+        <is>
+          <t>HALEU UMo 핵연료 초소형원자로에서 수소화이트륨 온도 궤환계수의 중성자 해석</t>
+        </is>
+      </c>
       <c r="D304" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -28384,7 +28736,11 @@
           <t>Oxygen substitution-induced structural, mechanical, and electronic evolution in UC1-xOx: A first-principles study for TRISO UCO fuel applications</t>
         </is>
       </c>
-      <c r="C305" s="9" t="inlineStr"/>
+      <c r="C305" s="9" t="inlineStr">
+        <is>
+          <t>UC1-xOx의 산소 치환에 따른 구조·기계·전자적 특성 변화: TRISO UCO 핵연료 적용을 위한 제1원리 연구</t>
+        </is>
+      </c>
       <c r="D305" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -28466,7 +28822,11 @@
           <t>Statistical admissibility of diffusion and SPN closures in correlated-medium nonclassical transport</t>
         </is>
       </c>
-      <c r="C306" s="9" t="inlineStr"/>
+      <c r="C306" s="9" t="inlineStr">
+        <is>
+          <t>상관 매질 비고전적 수송에서 확산 및 SPN 근사의 통계적 타당성</t>
+        </is>
+      </c>
       <c r="D306" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -28540,7 +28900,11 @@
           <t>Semi-mechanistic modeling of moisture release from heated concrete for safety design under sodium fire accident conditions</t>
         </is>
       </c>
-      <c r="C307" s="9" t="inlineStr"/>
+      <c r="C307" s="9" t="inlineStr">
+        <is>
+          <t>소듐 화재 사고 조건의 안전설계를 위한 가열 콘크리트의 수분 방출 반기계론적 모델링</t>
+        </is>
+      </c>
       <c r="D307" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -28622,7 +28986,11 @@
           <t>Comparative SRIM investigation of lutetium-based alloys and lead for alpha-particle shielding applications</t>
         </is>
       </c>
-      <c r="C308" s="9" t="inlineStr"/>
+      <c r="C308" s="9" t="inlineStr">
+        <is>
+          <t>알파입자 차폐 적용을 위한 루테튬 기반 합금과 납의 SRIM 비교 연구</t>
+        </is>
+      </c>
       <c r="D308" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -28704,7 +29072,11 @@
           <t>Experimental investigation of persistence spectra, spatial correlations, and vortex structures in a randomly packed pebble bed using time-resolved PIV</t>
         </is>
       </c>
-      <c r="C309" s="9" t="inlineStr"/>
+      <c r="C309" s="9" t="inlineStr">
+        <is>
+          <t>시간분해 PIV를 이용한 무작위 충전 페블베드 내 지속성 스펙트럼, 공간 상관 및 와류 구조 실험 연구</t>
+        </is>
+      </c>
       <c r="D309" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -28778,7 +29150,11 @@
           <t>Fuel cycle features of RFBB fast reactor with silicide fuel and lead coolant</t>
         </is>
       </c>
-      <c r="C310" s="9" t="inlineStr"/>
+      <c r="C310" s="9" t="inlineStr">
+        <is>
+          <t>규화물 핵연료 및 납 냉각재를 사용하는 RFBB 고속로의 핵연료주기 특성</t>
+        </is>
+      </c>
       <c r="D310" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -28860,7 +29236,11 @@
           <t>Monte Carlo investigation of spectral modifications induced by a W/Al selective filter in 6 MV flattening filter-free photon beams</t>
         </is>
       </c>
-      <c r="C311" s="9" t="inlineStr"/>
+      <c r="C311" s="9" t="inlineStr">
+        <is>
+          <t>6 MV 평탄화 필터 제거(FFF) 광자선에서 W/Al 선택 필터에 의한 스펙트럼 변화의 몬테카를로 연구</t>
+        </is>
+      </c>
       <c r="D311" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -28942,7 +29322,11 @@
           <t>Refined multiphysics coupling analysis in optimized isotope production</t>
         </is>
       </c>
-      <c r="C312" s="9" t="inlineStr"/>
+      <c r="C312" s="9" t="inlineStr">
+        <is>
+          <t>최적화된 동위원소 생산의 정밀 다중물리 연계 해석</t>
+        </is>
+      </c>
       <c r="D312" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -29024,7 +29408,11 @@
           <t>Core Deformation Reactivity Analysis Using a Neutronics–Thermal-Hydraulics–Structural Mechanics Coupled Method for FFTF LOFWOS TEST #13</t>
         </is>
       </c>
-      <c r="C313" s="9" t="inlineStr"/>
+      <c r="C313" s="9" t="inlineStr">
+        <is>
+          <t>FFTF LOFWOS TEST #13에 대한 중성자–열수력–구조역학 연계 방법을 이용한 노심 변형 반응도 해석</t>
+        </is>
+      </c>
       <c r="D313" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -29106,7 +29494,11 @@
           <t>Development and Deployment of a Machine Learning–Based Predictor of Moisture Carryover in Boiling Water Reactors</t>
         </is>
       </c>
-      <c r="C314" s="9" t="inlineStr"/>
+      <c r="C314" s="9" t="inlineStr">
+        <is>
+          <t>비등경수로 습분 이월 예측을 위한 기계학습 기반 예측기 개발 및 적용</t>
+        </is>
+      </c>
       <c r="D314" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -29188,7 +29580,11 @@
           <t>Insensitivity of scenario-based seismic fragility to distance-based inter-SSC correlation variations up to 1000 m in multi-unit NPPs</t>
         </is>
       </c>
-      <c r="C315" s="9" t="inlineStr"/>
+      <c r="C315" s="9" t="inlineStr">
+        <is>
+          <t>다수기 원자력발전소에서 1000 m 이내 거리 기반 SSC 간 상관관계 변화에 대한 시나리오 기반 지진 취약도의 둔감성</t>
+        </is>
+      </c>
       <c r="D315" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -29270,7 +29666,11 @@
           <t>Prediction of plutonium content of BWR/MOX fuel using a neural network</t>
         </is>
       </c>
-      <c r="C316" s="9" t="inlineStr"/>
+      <c r="C316" s="9" t="inlineStr">
+        <is>
+          <t>신경망을 이용한 BWR/MOX 핵연료의 플루토늄 함량 예측</t>
+        </is>
+      </c>
       <c r="D316" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -29352,7 +29752,11 @@
           <t>Experimental Characterization and Statistical Analysis of Two Geiger-Müller Detectors After Several Years of Use</t>
         </is>
       </c>
-      <c r="C317" s="9" t="inlineStr"/>
+      <c r="C317" s="9" t="inlineStr">
+        <is>
+          <t>수년간 사용한 두 가이거-뮐러 검출기의 실험적 특성 평가 및 통계 분석</t>
+        </is>
+      </c>
       <c r="D317" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -29434,7 +29838,11 @@
           <t>Analysis of natural deposition and spray removal characteristics of aerosols in containment based on PISAA code</t>
         </is>
       </c>
-      <c r="C318" s="9" t="inlineStr"/>
+      <c r="C318" s="9" t="inlineStr">
+        <is>
+          <t>PISAA 코드 기반 격납건물 내 에어로졸의 자연침적 및 살수 제거 특성 분석</t>
+        </is>
+      </c>
       <c r="D318" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -29516,7 +29924,11 @@
           <t>From data to correlation: symbolic regression reveals a unified friction factor relation for upward single-phase flow in vertical rod bundles</t>
         </is>
       </c>
-      <c r="C319" s="9" t="inlineStr"/>
+      <c r="C319" s="9" t="inlineStr">
+        <is>
+          <t>데이터에서 상관식으로: 기호회귀로 도출한 수직 봉다발 내 상향 단상유동의 통합 마찰계수 관계식</t>
+        </is>
+      </c>
       <c r="D319" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -29598,7 +30010,11 @@
           <t>Study of separation characteristics of corrugated-plate dryers under marine conditions</t>
         </is>
       </c>
-      <c r="C320" s="9" t="inlineStr"/>
+      <c r="C320" s="9" t="inlineStr">
+        <is>
+          <t>해양 조건에서 파형판 건조기의 분리 특성 연구</t>
+        </is>
+      </c>
       <c r="D320" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>
@@ -29680,7 +30096,11 @@
           <t>Predicting independent fission yields of the JEFF-4.0 evaluation via physics-informed machine learning surrogate models</t>
         </is>
       </c>
-      <c r="C321" s="9" t="inlineStr"/>
+      <c r="C321" s="9" t="inlineStr">
+        <is>
+          <t>물리정보 기계학습 대리모델을 이용한 JEFF-4.0 평가 독립 핵분열 수율 예측</t>
+        </is>
+      </c>
       <c r="D321" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -29754,7 +30174,11 @@
           <t>Scaling analysis of primary coolant system under SBLOCA for a test facility according to a pressurized water test reactor: Part I – top-down scaling</t>
         </is>
       </c>
-      <c r="C322" s="9" t="inlineStr"/>
+      <c r="C322" s="9" t="inlineStr">
+        <is>
+          <t>가압경수형 시험로 기반 시험장치의 SBLOCA 시 1차 냉각재계통 척도해석: 제1부 – 하향식 척도해석</t>
+        </is>
+      </c>
       <c r="D322" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -29836,7 +30260,11 @@
           <t>A simulation of the CAPRIX pin irradiation in comparison with experimental data: Illustration of the significance of accurate irradiation data</t>
         </is>
       </c>
-      <c r="C323" s="9" t="inlineStr"/>
+      <c r="C323" s="9" t="inlineStr">
+        <is>
+          <t>CAPRIX 연료봉 조사시험 모의 및 실험 데이터 비교: 정확한 조사 데이터의 중요성</t>
+        </is>
+      </c>
       <c r="D323" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -29910,7 +30338,11 @@
           <t>Numerical study on 7 to 61-rod LBE cooled wire-wrapped fuel rod bundles and the scalability to large-scale fuel assemblies</t>
         </is>
       </c>
-      <c r="C324" s="9" t="inlineStr"/>
+      <c r="C324" s="9" t="inlineStr">
+        <is>
+          <t>LBE 냉각 와이어랩 7~61봉 핵연료봉 다발의 수치해석 연구 및 대형 핵연료집합체로의 확장성</t>
+        </is>
+      </c>
       <c r="D324" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -29992,7 +30424,11 @@
           <t>An equivalent source response matrix method for solving the neutron diffusion equation</t>
         </is>
       </c>
-      <c r="C325" s="9" t="inlineStr"/>
+      <c r="C325" s="9" t="inlineStr">
+        <is>
+          <t>중성자 확산방정식 풀이를 위한 등가 선원 응답행렬 방법</t>
+        </is>
+      </c>
       <c r="D325" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -30074,7 +30510,11 @@
           <t>Applicability of regulatory Guide 1.99 Rev. 2 and ASTM E900-15 embrittlement trend curves to high-yield-strength RPV steels for small modular reactors</t>
         </is>
       </c>
-      <c r="C326" s="9" t="inlineStr"/>
+      <c r="C326" s="9" t="inlineStr">
+        <is>
+          <t>소형모듈원자로용 고항복강도 원자로압력용기강에 대한 Regulatory Guide 1.99 Rev. 2 및 ASTM E900-15 취화 경향 곡선의 적용성</t>
+        </is>
+      </c>
       <c r="D326" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -30156,7 +30596,11 @@
           <t>Investigation of the physicochemical responses and radical behavior of silk fabrics induced by gamma irradiation</t>
         </is>
       </c>
-      <c r="C327" s="9" t="inlineStr"/>
+      <c r="C327" s="9" t="inlineStr">
+        <is>
+          <t>감마선 조사에 따른 견직물의 물리화학적 반응 및 라디칼 거동 연구</t>
+        </is>
+      </c>
       <c r="D327" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -30230,7 +30674,11 @@
           <t>Removing oxygen-derived impurities from molten chloride fuel salts with aluminium chloride: Effectiveness and limitations</t>
         </is>
       </c>
-      <c r="C328" s="9" t="inlineStr"/>
+      <c r="C328" s="9" t="inlineStr">
+        <is>
+          <t>염화알루미늄을 이용한 용융 염화물 핵연료염 내 산소 유래 불순물 제거: 효과와 한계</t>
+        </is>
+      </c>
       <c r="D328" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -30304,7 +30752,11 @@
           <t>Comprehensive validation of subchannel analysis code SACOS-LMR with liquid-sodium and -lead benchmarks</t>
         </is>
       </c>
-      <c r="C329" s="9" t="inlineStr"/>
+      <c r="C329" s="9" t="inlineStr">
+        <is>
+          <t>액체 소듐 및 납 벤치마크를 이용한 부수로 해석코드 SACOS-LMR의 종합 검증</t>
+        </is>
+      </c>
       <c r="D329" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -30386,7 +30838,11 @@
           <t>Innovative techniques in evaluating neutron fluxes of the multi-energy groups diffusion for homogeneous cubic and spherical reactors</t>
         </is>
       </c>
-      <c r="C330" s="9" t="inlineStr"/>
+      <c r="C330" s="9" t="inlineStr">
+        <is>
+          <t>균질 입방체 및 구형 원자로에 대한 다군 확산 중성자속 평가의 혁신적 기법</t>
+        </is>
+      </c>
       <c r="D330" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -30468,7 +30924,11 @@
           <t>Radiological site evaluation of the proposed Gosong Beach nuclear power plant site in Indonesia</t>
         </is>
       </c>
-      <c r="C331" s="9" t="inlineStr"/>
+      <c r="C331" s="9" t="inlineStr">
+        <is>
+          <t>인도네시아 고송 해변 원자력발전소 후보 부지의 방사선학적 부지 평가</t>
+        </is>
+      </c>
       <c r="D331" t="inlineStr">
         <is>
           <t>Annals of Nuclear Energy</t>
@@ -30550,7 +31010,11 @@
           <t>Coupled flow-thermal analysis of an HTGR spent fuel dry storage system during transfer and storage</t>
         </is>
       </c>
-      <c r="C332" s="9" t="inlineStr"/>
+      <c r="C332" s="9" t="inlineStr">
+        <is>
+          <t>HTGR 사용후핵연료 건식저장계통의 이송 및 저장 중 유동-열 연계 해석</t>
+        </is>
+      </c>
       <c r="D332" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -30632,7 +31096,11 @@
           <t>Design and analysis of a bedrock-coupled passive heat removal system for a small modular reactor</t>
         </is>
       </c>
-      <c r="C333" s="9" t="inlineStr"/>
+      <c r="C333" s="9" t="inlineStr">
+        <is>
+          <t>소형모듈원자로용 암반 연계 피동열제거계통 설계 및 해석</t>
+        </is>
+      </c>
       <c r="D333" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Design</t>
@@ -30706,7 +31174,11 @@
           <t>An uncertainty-aware machine learning framework for predicting cable and cabinet damage in switchgear room fire scenarios</t>
         </is>
       </c>
-      <c r="C334" s="9" t="inlineStr"/>
+      <c r="C334" s="9" t="inlineStr">
+        <is>
+          <t>개폐기실 화재 시나리오에서 케이블 및 캐비닛 손상 예측을 위한 불확실성 인지 기계학습 프레임워크</t>
+        </is>
+      </c>
       <c r="D334" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -30788,7 +31260,11 @@
           <t>Analysis of low-level alarm for a lubricating oil tank based on flow characteristics and temperature in a nuclear power plant</t>
         </is>
       </c>
-      <c r="C335" s="9" t="inlineStr"/>
+      <c r="C335" s="9" t="inlineStr">
+        <is>
+          <t>원자력발전소 윤활유 탱크의 유동 특성 및 온도 기반 저수위 경보 분석</t>
+        </is>
+      </c>
       <c r="D335" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -30870,7 +31346,11 @@
           <t>Computational assessment of the feasibility of conversion of the impulse graphite reactor to high-assay low-enriched uranium fuel</t>
         </is>
       </c>
-      <c r="C336" s="9" t="inlineStr"/>
+      <c r="C336" s="9" t="inlineStr">
+        <is>
+          <t>임펄스 흑연원자로의 HALEU 핵연료 전환 타당성에 대한 전산 평가</t>
+        </is>
+      </c>
       <c r="D336" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -30944,7 +31424,11 @@
           <t>Investigation into peak shaving technology for nuclear power systems utilizing SOEC technology</t>
         </is>
       </c>
-      <c r="C337" s="9" t="inlineStr"/>
+      <c r="C337" s="9" t="inlineStr">
+        <is>
+          <t>SOEC 기술을 활용한 원자력 계통의 첨두부하 저감 기술 연구</t>
+        </is>
+      </c>
       <c r="D337" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -31026,7 +31510,11 @@
           <t>Local lattice distortion-induced mechanical asymmetry and coupled magnetic-electronic responses in bcc iron: A combined experimental and first-principles investigation</t>
         </is>
       </c>
-      <c r="C338" s="9" t="inlineStr"/>
+      <c r="C338" s="9" t="inlineStr">
+        <is>
+          <t>bcc 철에서 국부 격자 뒤틀림에 의한 기계적 비대칭성과 자기-전자 연계 반응: 실험 및 제1원리 복합 연구</t>
+        </is>
+      </c>
       <c r="D338" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -31108,7 +31596,11 @@
           <t>Neutron leakage spectra benchmark of spherical iron sample with a 252Cf fission source</t>
         </is>
       </c>
-      <c r="C339" s="9" t="inlineStr"/>
+      <c r="C339" s="9" t="inlineStr">
+        <is>
+          <t>252Cf 핵분열 선원을 이용한 구형 철 시료의 중성자 누설 스펙트럼 벤치마크</t>
+        </is>
+      </c>
       <c r="D339" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -31182,7 +31674,11 @@
           <t>Regulatory readiness for SMRs in Greece: An institutional gap analysis of a latent EU newcomer</t>
         </is>
       </c>
-      <c r="C340" s="9" t="inlineStr"/>
+      <c r="C340" s="9" t="inlineStr">
+        <is>
+          <t>그리스의 SMR 규제 준비도: 잠재적 EU 신규 도입국의 제도적 격차 분석</t>
+        </is>
+      </c>
       <c r="D340" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -31264,7 +31760,11 @@
           <t>Strontium-90 determination in milk ash by cherenkov and gas-flow proportional counting: A comparison of three radiochemical separations</t>
         </is>
       </c>
-      <c r="C341" s="9" t="inlineStr"/>
+      <c r="C341" s="9" t="inlineStr">
+        <is>
+          <t>체렌코프 계수 및 기체유동 비례계수를 이용한 우유 회분 중 스트론튬-90 정량: 세 가지 방사화학적 분리법 비교</t>
+        </is>
+      </c>
       <c r="D341" t="inlineStr">
         <is>
           <t>Nuclear Engineering and Technology</t>
@@ -31338,7 +31838,11 @@
           <t>Balance of Plant Modeling and Real-Time Hardware-in-the-Loop Integration with the Microreactor Automated Control System</t>
         </is>
       </c>
-      <c r="C342" s="9" t="inlineStr"/>
+      <c r="C342" s="9" t="inlineStr">
+        <is>
+          <t>BOP 모델링 및 초소형원자로 자동제어계통과의 실시간 HIL(Hardware-in-the-Loop) 통합</t>
+        </is>
+      </c>
       <c r="D342" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -31420,7 +31924,11 @@
           <t>Evaluation of Neutron-Induced Radiation Generated by a Vehicle-Mounted System for Hazardous Material Detection</t>
         </is>
       </c>
-      <c r="C343" s="9" t="inlineStr"/>
+      <c r="C343" s="9" t="inlineStr">
+        <is>
+          <t>유해물질 탐지용 차량 탑재 시스템에서 발생하는 중성자 유발 방사선 평가</t>
+        </is>
+      </c>
       <c r="D343" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -31502,7 +32010,11 @@
           <t>Reliability Analysis and 30 Years of Operational Performance of the GHARR-1 Control Rod System</t>
         </is>
       </c>
-      <c r="C344" s="9" t="inlineStr"/>
+      <c r="C344" s="9" t="inlineStr">
+        <is>
+          <t>GHARR-1 제어봉 계통의 신뢰도 분석 및 30년 운전 성능</t>
+        </is>
+      </c>
       <c r="D344" t="inlineStr">
         <is>
           <t>Nuclear Technology</t>
@@ -31584,7 +32096,11 @@
           <t>Experimental and numerical study of the formation and breakdown of density stratification in an air-steam containment atmosphere with internal cooler and steam injection</t>
         </is>
       </c>
-      <c r="C345" s="9" t="inlineStr"/>
+      <c r="C345" s="9" t="inlineStr">
+        <is>
+          <t>내부 냉각기 및 증기 주입이 있는 공기-증기 격납건물 대기에서 밀도 성층의 형성 및 붕괴에 관한 실험 및 수치해석 연구</t>
+        </is>
+      </c>
       <c r="D345" t="inlineStr">
         <is>
           <t>Progress in Nuclear Energy</t>

</xml_diff>

<commit_message>
Expand translation corrections and apply them to earlier machine translations
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sHSCbWkWUBv2qJdcCnH5x
</commit_message>
<xml_diff>
--- a/outputs/nuclear-literature-database.xlsx
+++ b/outputs/nuclear-literature-database.xlsx
@@ -1576,7 +1576,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>직접 수치 시뮬레이션 (DNS) 을 사용하여 베어로드 번들 하위 채널의 무한한 배열의 기하학적 표현에 대한 조사</t>
+          <t>직접 수치 시뮬레이션 (DNS) 을 사용하여 베어로드 번들 부수로의 무한한 배열의 기하학적 표현에 대한 조사</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>코어 내 계측 루프를 위한 배포 지향 단일 채널 무결성 평가 및 장애 하위 유형 분류 프레임워크</t>
+          <t>노내 계측 루프를 위한 배포 지향 단일 채널 무결성 평가 및 장애 하위 유형 분류 프레임워크</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>원자력 발전소 장비의 알 수 없는 결함 진단을 위한 이전 학습 지원 비지도 클러스터링 접근법</t>
+          <t>원자력 발전소 장비의 알 수 없는 결함 진단을 위한 전이학습 지원 비지도 클러스터링 접근법</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>페블 베드 원자로에서 다단계 텔레스코픽 제어 로드 평가, 파트 I: 기계 설계, 중성 평가 및 경제 분석</t>
+          <t>페블베드 원자로에서 다단계 텔레스코픽 제어봉 평가, 파트 I: 기계 설계, 중성 평가 및 경제 분석</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>HTR-10의 1차 회로에서 삼중수소 활성을 갖는 붕소 함유 침착물: 실험적 측정 및 원천 분석</t>
+          <t>HTR-10의 1차 계통에서 삼중수소 활성을 갖는 붕소 함유 침착물: 실험적 측정 및 원천 분석</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>NPP에서 대규모 장애 트리 중요도 분석을 위한 GPU 병렬화 방법에 대한 연구</t>
+          <t>NPP에서 대규모 고장수목 중요도 분석을 위한 GPU 병렬화 방법에 대한 연구</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>OpenMC에서 고갈 사슬 파일이 동위원소 예측 정확도에 미치는 영향: SFCOMPO 데이터를 이용한 후쿠시마 다이니 1호기 BWR 분석</t>
+          <t>OpenMC에서 연소 체인 파일이 동위원소 예측 정확도에 미치는 영향: SFCOMPO 데이터를 이용한 후쿠시마 다이니 1호기 BWR 분석</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>다중 데이터 세트를 사용한 세라믹 핵 연료의 분열 가스 방출 및 팽윤을 위한 미세 분해 및 미세 구조적 진화의 물리 기반 모델 평가</t>
+          <t>다중 데이터 세트를 사용한 세라믹 핵 연료의 핵분열기체 방출 및 팽윤을 위한 미세 분해 및 미세 구조적 진화의 물리 기반 모델 평가</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>U-Mo 연료에 대한 DART 코드에서 분열 가스 매개변수의 기계 학습 지원 보정</t>
+          <t>U-Mo 연료에 대한 DART 코드에서 핵분열기체 매개변수의 기계 학습 지원 보정</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>HPR1000에서 대체 소스 용어 평가를 위한 PSA 정보에 입각한 방법론</t>
+          <t>HPR1000에서 대체 선원항 평가를 위한 PSA 정보에 입각한 방법론</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>자갈층 원자로 분석을 위한 뉴트로닉스, 이산소자법, 열수력 및 보로노이 메쉬의 커플링</t>
+          <t>페블베드 원자로 분석을 위한 중성자 해석, 이산소자법, 열수력 및 보로노이 메쉬의 커플링</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>용융염 원자로 분석을 위한 지속적인 재처리 및 연료 유동을 고려한 고갈도 계산 방법 개발</t>
+          <t>용융염 원자로 분석을 위한 지속적인 재처리 및 연료 유동을 고려한 연소 계산 방법 개발</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>유체 대 유체 자연 순환 루프에서 유동 및 열 전달 특성의 유사성 분석</t>
+          <t>Fluid-to-Fluid 자연 순환 루프에서 유동 및 열전달 특성의 유사성 분석</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>미래 에너지 시스템의 소형 모듈식 원자로: 계통 지원, 분산형 에너지 시스템, 비전기 응용 분야 및 경제 동인에 대한 연구</t>
+          <t>미래 에너지 시스템의 소형모듈원자로(SMR): 계통 지원, 분산형 에너지 시스템, 비전기 응용 분야 및 경제 동인에 대한 연구</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>RIA와 동등한 열팽창 하중 하에서 전체 UO2 연료 펠릿의 손상 진화에 대한 주변 평가</t>
+          <t>RIA와 동등한 열팽창 하중 하에서 전체 UO2 핵연료 소결체의 손상 진화에 대한 주변 평가</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -4556,7 +4556,7 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>정상 상태 PWR 조건에서 Cr 코팅 사고 내성 연료의 열 마진에 대한 포괄적 분석</t>
+          <t>정상 상태 PWR 조건에서 Cr 코팅 사고저항성핵연료(ATF)의 열적 여유도에 대한 포괄적 분석</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4642,7 +4642,7 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>인공 신경망 지원 프레임워크를 사용하여 아냉각 유동 비등에서 핵산 비등 열속으로부터의 이탈 예측에 대한 상관 관계 개발</t>
+          <t>인공 신경망 지원 프레임워크를 사용하여 아냉각 유동 비등에서 핵비등 열속으로부터의 이탈 예측에 대한 상관 관계 개발</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>표면 오염 측정을 위한 2D 슬램 기반 방사선 매핑 시스템 개발</t>
+          <t>표면 오염 측정을 위한 2D SLAM 기반 방사선 매핑 시스템 개발</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>핵 비상 대응에서 그룹화된 소스 용어 예측을 위한 순방향 앙상블 머신 러닝</t>
+          <t>핵 비상 대응에서 그룹화된 선원항 예측을 위한 순방향 앙상블 머신 러닝</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>다중 구획 격납 장치에서 PCS 구동 자연 순환 및 증기 층화에 대한 개구 기하학의 상호 연결 효과에 대한 수치 연구</t>
+          <t>다중 구획 격납건물에서 PCS 구동 자연 순환 및 증기 층화에 대한 개구 기하학의 상호 연결 효과에 대한 수치 연구</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -5550,7 +5550,7 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>개념 제안: 고온의 나트륨 증기로 냉각된 원자로</t>
+          <t>개념 제안: 고온의 소듐 증기로 냉각된 원자로</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -5644,7 +5644,7 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>지출된 TRISO 연료를 위한 OpenMC 고정 소스 중성자 전송 시뮬레이션을 사용한 다중 그룹 단면 생성</t>
+          <t>사용후 TRISO 연료를 위한 OpenMC 고정 소스 중성자 수송 시뮬레이션을 사용한 다군 단면적 생성</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>자갈층 기하학에서 He-Xe 및 He-Kr 이진 혼합물의 열수력 성능에 대한 수치 상관 관계</t>
+          <t>페블베드 기하학에서 He-Xe 및 He-Kr 이진 혼합물의 열수력 성능에 대한 수치 상관 관계</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>제한된 측정 샘플을 사용하여 핵연료봉의 유동유발 진동 예측을 위한 신규 부품 모드 합성-정규 직교 분해-감소-차수 모델</t>
+          <t>제한된 측정 샘플을 사용하여 핵연료봉의 유동유발진동 예측을 위한 신규 부품 모드 합성-정규 직교 분해-감소-차수 모델</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>수치 시뮬레이션을 통한 발산 컨버징 나트륨 히트 파이프의 구조 설계 및 열전달 성능 연구</t>
+          <t>수치 시뮬레이션을 통한 발산 컨버징 소듐 히트 파이프의 구조 설계 및 열전달 성능 연구</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>원자력 발전소의 복합 사건에 대한 동적 위험 평가를 위해 격실 기반 유압 홍수 전파와 지진 취약성 통합</t>
+          <t>원자력 발전소의 복합 사건에 대한 동적 위험 평가를 위해 격실 기반 침수 전파와 지진 취약성 통합</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -6796,7 +6796,7 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>지질 저장소의 열-수력 커플링 환경에 노출된 탄소섬유 강화 벤토나이트의 건조 균열 및 미세구조 변화에 대한 실험실 평가</t>
+          <t>지층처분장의 열-수력 커플링 환경에 노출된 탄소섬유 강화 벤토나이트의 건조 균열 및 미세구조 변화에 대한 실험실 평가</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -7094,7 +7094,7 @@
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>ETRR-2에서의 가상의 사고에 대한 방사능 방출의 원천 용어 및 예측 분석</t>
+          <t>ETRR-2에서의 가상의 사고에 대한 방사능 방출의 선원항 및 예측 분석</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>나선형 십자형 핵연료봉 번들에 데이터 구동 포드 감소 주문 모델 적용</t>
+          <t>나선형 십자형 핵연료봉 번들에 데이터 구동 POD 차수축소모델 적용</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>광고에서 237NpTransmutation 고갈의 베이지안 최적화 기반 기계 학습 반전</t>
+          <t>ADS에서 237NpTransmutation 연소의 베이지안 최적화 기반 기계 학습 반전</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -7580,7 +7580,7 @@
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>핵연료에서 높은 연소 구조 형성에 대한 모델링: 기포 압력 기반 접근법</t>
+          <t>핵연료에서 고연소도 조직 형성에 대한 모델링: 기포 압력 기반 접근법</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7666,7 +7666,7 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>사용후핵연료에서 에너지-선택적 변이에 대한 이론적 평가</t>
+          <t>사용후핵연료에서 에너지-선택적 핵변환에 대한 이론적 평가</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">

</xml_diff>

<commit_message>
Weekly digest 2026-09-21 success
</commit_message>
<xml_diff>
--- a/outputs/nuclear-literature-database.xlsx
+++ b/outputs/nuclear-literature-database.xlsx
@@ -38742,17 +38742,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-23T10:18:44</t>
+          <t>2026-09-23T10:21:04</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>67</v>
       </c>
       <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
         <v>67</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>

</xml_diff>